<commit_message>
W34 2026 weekly update
- 本周标的+票息, 重生成 watchlist.json(54只, 带ko/敲入类型/板块热点图)
- 修复: generate_watchlist 模型 deepseek-v4-pro→deepseek-chat(v4-pro服务端变推理模型、content返回空)
- 财经日历刷新至W34(回顾8/10-14 CPI+3.4%/PPI持平/零售-0.6%/AMAT超预期; 预告FOMC纪要8/19/JacksonHole8/27-29/NVDA8/26)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/低波精选组.xlsx
+++ b/低波精选组.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Y:\GopherHK\Fixed Income\结构化产品\HTML 生成\FCN_Watchlist_交接\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F74CE01-E2F7-4DC6-A4AA-B3DF0B783499}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6FABCB4-F387-4EF2-B60E-D56034769E81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="68">
   <si>
     <t>区域</t>
   </si>
@@ -52,6 +52,18 @@
     <t>港股</t>
   </si>
   <si>
+    <t>2359 HK</t>
+  </si>
+  <si>
+    <t>药明康德</t>
+  </si>
+  <si>
+    <t>Diagnostics &amp; Research</t>
+  </si>
+  <si>
+    <t>欧式敲入</t>
+  </si>
+  <si>
     <t>3808 HK</t>
   </si>
   <si>
@@ -61,16 +73,13 @@
     <t>Farm &amp; Heavy Construction Machinery</t>
   </si>
   <si>
-    <t>欧式敲入</t>
-  </si>
-  <si>
-    <t>2359 HK</t>
-  </si>
-  <si>
-    <t>药明康德</t>
-  </si>
-  <si>
-    <t>Diagnostics &amp; Research</t>
+    <t>9988 HK</t>
+  </si>
+  <si>
+    <t>阿里巴巴</t>
+  </si>
+  <si>
+    <t>电商/云</t>
   </si>
   <si>
     <t>2382 HK</t>
@@ -82,15 +91,6 @@
     <t>光学/AI硬件</t>
   </si>
   <si>
-    <t>9988 HK</t>
-  </si>
-  <si>
-    <t>阿里巴巴</t>
-  </si>
-  <si>
-    <t>电商/云</t>
-  </si>
-  <si>
     <t>1024 HK</t>
   </si>
   <si>
@@ -121,13 +121,49 @@
     <t>Electronic Components</t>
   </si>
   <si>
-    <t>CSCO US</t>
-  </si>
-  <si>
-    <t>思科</t>
-  </si>
-  <si>
-    <t>Communication Equipment</t>
+    <t>ASML US</t>
+  </si>
+  <si>
+    <t>阿斯麦</t>
+  </si>
+  <si>
+    <t>半导体设备</t>
+  </si>
+  <si>
+    <t>PLTR US</t>
+  </si>
+  <si>
+    <t>Palantir</t>
+  </si>
+  <si>
+    <t>AI软件</t>
+  </si>
+  <si>
+    <t>NU US</t>
+  </si>
+  <si>
+    <t>Nu Holdings</t>
+  </si>
+  <si>
+    <t>Banks - Regional</t>
+  </si>
+  <si>
+    <t>TSM US</t>
+  </si>
+  <si>
+    <t>台积电ADR</t>
+  </si>
+  <si>
+    <t>晶圆代工</t>
+  </si>
+  <si>
+    <t>FDX US</t>
+  </si>
+  <si>
+    <t>联邦快递</t>
+  </si>
+  <si>
+    <t>Integrated Freight &amp; Logistics</t>
   </si>
   <si>
     <t>AVGO US</t>
@@ -139,63 +175,42 @@
     <t>半导体</t>
   </si>
   <si>
+    <t>GEV US</t>
+  </si>
+  <si>
+    <t>GE Vernova</t>
+  </si>
+  <si>
+    <t>Specialty Industrial Machinery</t>
+  </si>
+  <si>
+    <t>CRM US</t>
+  </si>
+  <si>
+    <t>赛富时</t>
+  </si>
+  <si>
+    <t>Software - Application</t>
+  </si>
+  <si>
+    <t>NOW US</t>
+  </si>
+  <si>
+    <t>ServiceNow</t>
+  </si>
+  <si>
     <t>WDAY US</t>
   </si>
   <si>
     <t>Workday</t>
   </si>
   <si>
-    <t>Software - Application</t>
-  </si>
-  <si>
-    <t>ASML US</t>
-  </si>
-  <si>
-    <t>阿斯麦</t>
-  </si>
-  <si>
-    <t>半导体设备</t>
-  </si>
-  <si>
-    <t>RCL US</t>
-  </si>
-  <si>
-    <t>皇家加勒比邮轮</t>
-  </si>
-  <si>
-    <t>Travel Services</t>
-  </si>
-  <si>
-    <t>NVDA US</t>
-  </si>
-  <si>
-    <t>英伟达</t>
-  </si>
-  <si>
-    <t>AI芯片</t>
-  </si>
-  <si>
     <t>SPOT US</t>
   </si>
   <si>
     <t>Spotify Technology</t>
   </si>
   <si>
-    <t>TSM US</t>
-  </si>
-  <si>
-    <t>台积电ADR</t>
-  </si>
-  <si>
-    <t>晶圆代工</t>
-  </si>
-  <si>
-    <t>CRM US</t>
-  </si>
-  <si>
-    <t>赛富时</t>
-  </si>
-  <si>
     <t>ADI US</t>
   </si>
   <si>
@@ -205,28 +220,10 @@
     <t>Semiconductors</t>
   </si>
   <si>
-    <t>NU US</t>
-  </si>
-  <si>
-    <t>Nu Holdings</t>
-  </si>
-  <si>
-    <t>Banks - Regional</t>
-  </si>
-  <si>
-    <t>FDX US</t>
-  </si>
-  <si>
-    <t>联邦快递</t>
-  </si>
-  <si>
-    <t>Integrated Freight &amp; Logistics</t>
-  </si>
-  <si>
-    <t>NXPI US</t>
-  </si>
-  <si>
-    <t>恩智浦</t>
+    <t>MCHP US</t>
+  </si>
+  <si>
+    <t>微芯科技</t>
   </si>
 </sst>
 </file>
@@ -632,7 +629,7 @@
         <v>1.01</v>
       </c>
       <c r="I2" s="1">
-        <v>8.9099999999999999E-2</v>
+        <v>0.14940000000000001</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.15">
@@ -649,10 +646,10 @@
         <v>16</v>
       </c>
       <c r="E3">
-        <v>0.81</v>
+        <v>0.8</v>
       </c>
       <c r="F3">
-        <v>0.71</v>
+        <v>0.7</v>
       </c>
       <c r="G3" t="s">
         <v>13</v>
@@ -661,7 +658,7 @@
         <v>1.01</v>
       </c>
       <c r="I3" s="1">
-        <v>0.14430000000000001</v>
+        <v>8.8900000000000007E-2</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.15">
@@ -678,10 +675,10 @@
         <v>19</v>
       </c>
       <c r="E4">
-        <v>0.84</v>
+        <v>0.85</v>
       </c>
       <c r="F4">
-        <v>0.74</v>
+        <v>0.75</v>
       </c>
       <c r="G4" t="s">
         <v>13</v>
@@ -690,7 +687,7 @@
         <v>1.01</v>
       </c>
       <c r="I4" s="1">
-        <v>0.20100000000000001</v>
+        <v>0.1419</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.15">
@@ -707,10 +704,10 @@
         <v>22</v>
       </c>
       <c r="E5">
-        <v>0.85</v>
+        <v>0.8</v>
       </c>
       <c r="F5">
-        <v>0.75</v>
+        <v>0.7</v>
       </c>
       <c r="G5" t="s">
         <v>13</v>
@@ -719,7 +716,7 @@
         <v>1.01</v>
       </c>
       <c r="I5" s="1">
-        <v>0.15359999999999999</v>
+        <v>0.14940000000000001</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.15">
@@ -748,7 +745,7 @@
         <v>1.01</v>
       </c>
       <c r="I6" s="1">
-        <v>0.15590000000000001</v>
+        <v>0.1459</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.15">
@@ -765,10 +762,10 @@
         <v>28</v>
       </c>
       <c r="E7">
-        <v>0.82</v>
+        <v>0.83</v>
       </c>
       <c r="F7">
-        <v>0.72</v>
+        <v>0.73</v>
       </c>
       <c r="G7" t="s">
         <v>13</v>
@@ -777,7 +774,7 @@
         <v>1.01</v>
       </c>
       <c r="I7" s="1">
-        <v>0.19350000000000001</v>
+        <v>0.2064</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.15">
@@ -794,10 +791,10 @@
         <v>32</v>
       </c>
       <c r="E8">
-        <v>0.84</v>
+        <v>0.82</v>
       </c>
       <c r="F8">
-        <v>0.74</v>
+        <v>0.72</v>
       </c>
       <c r="G8" t="s">
         <v>13</v>
@@ -806,7 +803,7 @@
         <v>1.01</v>
       </c>
       <c r="I8" s="1">
-        <v>0.1875</v>
+        <v>0.14979999999999999</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.15">
@@ -823,10 +820,10 @@
         <v>35</v>
       </c>
       <c r="E9">
-        <v>0.85</v>
+        <v>0.79</v>
       </c>
       <c r="F9">
-        <v>0.75</v>
+        <v>0.69</v>
       </c>
       <c r="G9" t="s">
         <v>13</v>
@@ -835,7 +832,7 @@
         <v>1.01</v>
       </c>
       <c r="I9" s="1">
-        <v>0.14050000000000001</v>
+        <v>0.15340000000000001</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.15">
@@ -852,10 +849,10 @@
         <v>38</v>
       </c>
       <c r="E10">
-        <v>0.79</v>
+        <v>0.82</v>
       </c>
       <c r="F10">
-        <v>0.69</v>
+        <v>0.72</v>
       </c>
       <c r="G10" t="s">
         <v>13</v>
@@ -864,7 +861,7 @@
         <v>1.01</v>
       </c>
       <c r="I10" s="1">
-        <v>0.1447</v>
+        <v>0.2051</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.15">
@@ -881,10 +878,10 @@
         <v>41</v>
       </c>
       <c r="E11">
-        <v>0.76</v>
+        <v>0.85</v>
       </c>
       <c r="F11">
-        <v>0.66</v>
+        <v>0.75</v>
       </c>
       <c r="G11" t="s">
         <v>13</v>
@@ -893,7 +890,7 @@
         <v>1.01</v>
       </c>
       <c r="I11" s="1">
-        <v>0.20250000000000001</v>
+        <v>0.1235</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.15">
@@ -910,10 +907,10 @@
         <v>44</v>
       </c>
       <c r="E12">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="F12">
-        <v>0.72</v>
+        <v>0.75</v>
       </c>
       <c r="G12" t="s">
         <v>13</v>
@@ -922,7 +919,7 @@
         <v>1.01</v>
       </c>
       <c r="I12" s="1">
-        <v>0.19620000000000001</v>
+        <v>0.13689999999999999</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.15">
@@ -939,10 +936,10 @@
         <v>47</v>
       </c>
       <c r="E13">
-        <v>0.83</v>
+        <v>0.85</v>
       </c>
       <c r="F13">
-        <v>0.73</v>
+        <v>0.75</v>
       </c>
       <c r="G13" t="s">
         <v>13</v>
@@ -951,7 +948,7 @@
         <v>1.01</v>
       </c>
       <c r="I13" s="1">
-        <v>0.14649999999999999</v>
+        <v>7.6600000000000001E-2</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.15">
@@ -968,10 +965,10 @@
         <v>50</v>
       </c>
       <c r="E14">
-        <v>0.85</v>
+        <v>0.82</v>
       </c>
       <c r="F14">
-        <v>0.75</v>
+        <v>0.72</v>
       </c>
       <c r="G14" t="s">
         <v>13</v>
@@ -980,7 +977,7 @@
         <v>1.01</v>
       </c>
       <c r="I14" s="1">
-        <v>0.13730000000000001</v>
+        <v>0.15049999999999999</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.15">
@@ -994,13 +991,13 @@
         <v>52</v>
       </c>
       <c r="D15" t="s">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="E15">
-        <v>0.85</v>
+        <v>0.83</v>
       </c>
       <c r="F15">
-        <v>0.75</v>
+        <v>0.73</v>
       </c>
       <c r="G15" t="s">
         <v>13</v>
@@ -1009,7 +1006,7 @@
         <v>1.01</v>
       </c>
       <c r="I15" s="1">
-        <v>0.14230000000000001</v>
+        <v>0.19009999999999999</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.15">
@@ -1017,13 +1014,13 @@
         <v>29</v>
       </c>
       <c r="B16" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C16" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D16" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E16">
         <v>0.84</v>
@@ -1038,7 +1035,7 @@
         <v>1.01</v>
       </c>
       <c r="I16" s="1">
-        <v>0.13589999999999999</v>
+        <v>0.15190000000000001</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.15">
@@ -1046,19 +1043,19 @@
         <v>29</v>
       </c>
       <c r="B17" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C17" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D17" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E17">
-        <v>0.82</v>
+        <v>0.81</v>
       </c>
       <c r="F17">
-        <v>0.72</v>
+        <v>0.71</v>
       </c>
       <c r="G17" t="s">
         <v>13</v>
@@ -1067,7 +1064,7 @@
         <v>1.01</v>
       </c>
       <c r="I17" s="1">
-        <v>0.1447</v>
+        <v>0.2026</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.15">
@@ -1075,19 +1072,19 @@
         <v>29</v>
       </c>
       <c r="B18" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C18" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D18" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="E18">
-        <v>0.8</v>
+        <v>0.83</v>
       </c>
       <c r="F18">
-        <v>0.7</v>
+        <v>0.73</v>
       </c>
       <c r="G18" t="s">
         <v>13</v>
@@ -1096,7 +1093,7 @@
         <v>1.01</v>
       </c>
       <c r="I18" s="1">
-        <v>0.15079999999999999</v>
+        <v>0.1487</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.15">
@@ -1110,13 +1107,13 @@
         <v>62</v>
       </c>
       <c r="D19" t="s">
-        <v>63</v>
+        <v>25</v>
       </c>
       <c r="E19">
-        <v>0.83</v>
+        <v>0.85</v>
       </c>
       <c r="F19">
-        <v>0.73</v>
+        <v>0.75</v>
       </c>
       <c r="G19" t="s">
         <v>13</v>
@@ -1125,7 +1122,7 @@
         <v>1.01</v>
       </c>
       <c r="I19" s="1">
-        <v>0.14380000000000001</v>
+        <v>0.1522</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.15">
@@ -1133,19 +1130,19 @@
         <v>29</v>
       </c>
       <c r="B20" t="s">
+        <v>63</v>
+      </c>
+      <c r="C20" t="s">
         <v>64</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
         <v>65</v>
       </c>
-      <c r="D20" t="s">
-        <v>66</v>
-      </c>
       <c r="E20">
-        <v>0.85</v>
+        <v>0.83</v>
       </c>
       <c r="F20">
-        <v>0.75</v>
+        <v>0.73</v>
       </c>
       <c r="G20" t="s">
         <v>13</v>
@@ -1154,7 +1151,7 @@
         <v>1.01</v>
       </c>
       <c r="I20" s="1">
-        <v>7.2300000000000003E-2</v>
+        <v>0.1404</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.15">
@@ -1162,13 +1159,13 @@
         <v>29</v>
       </c>
       <c r="B21" t="s">
+        <v>66</v>
+      </c>
+      <c r="C21" t="s">
         <v>67</v>
       </c>
-      <c r="C21" t="s">
-        <v>68</v>
-      </c>
       <c r="D21" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="E21">
         <v>0.82</v>
@@ -1183,7 +1180,7 @@
         <v>1.01</v>
       </c>
       <c r="I21" s="1">
-        <v>0.19550000000000001</v>
+        <v>0.19700000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
W39 2026 weekly update
- 本周标的+票息, 名称/行业自动中文, 重生成 watchlist.json(51只, 无NaN)
- 财经日历刷新至W39(回顾FOMC 9/16加息25bp至3.75-4.00%2023来首次; 预告核心PCE9/30·美光9/30·埃森哲10/1·非农10/2)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/低波精选组.xlsx
+++ b/低波精选组.xlsx
@@ -8,19 +8,32 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Y:\GopherHK\Fixed Income\结构化产品\HTML 生成\FCN_Watchlist_交接\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC0847FE-CF9E-4006-AE35-29ECD523F667}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE1733EE-2FCB-4A10-A70A-D28DD1CCF502}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="68">
   <si>
     <t>区域</t>
   </si>
@@ -52,6 +65,18 @@
     <t>港股</t>
   </si>
   <si>
+    <t>1093 HK</t>
+  </si>
+  <si>
+    <t>石药集团</t>
+  </si>
+  <si>
+    <t>制药</t>
+  </si>
+  <si>
+    <t>欧式敲入</t>
+  </si>
+  <si>
     <t>2359 HK</t>
   </si>
   <si>
@@ -61,64 +86,100 @@
     <t>诊断与研究</t>
   </si>
   <si>
-    <t>欧式敲入</t>
-  </si>
-  <si>
-    <t>2899 HK</t>
-  </si>
-  <si>
-    <t>紫金矿业</t>
+    <t>2382 HK</t>
+  </si>
+  <si>
+    <t>舜宇光学</t>
+  </si>
+  <si>
+    <t>光学/AI硬件</t>
+  </si>
+  <si>
+    <t>9988 HK</t>
+  </si>
+  <si>
+    <t>阿里巴巴</t>
+  </si>
+  <si>
+    <t>电商/云</t>
+  </si>
+  <si>
+    <t>1024 HK</t>
+  </si>
+  <si>
+    <t>快手-W</t>
+  </si>
+  <si>
+    <t>互联网内容与信息</t>
+  </si>
+  <si>
+    <t>1810 HK</t>
+  </si>
+  <si>
+    <t>小米集团</t>
+  </si>
+  <si>
+    <t>AI/IoT</t>
+  </si>
+  <si>
+    <t>美股</t>
+  </si>
+  <si>
+    <t>ANET US</t>
+  </si>
+  <si>
+    <t>阿里斯塔</t>
+  </si>
+  <si>
+    <t>AI网络</t>
+  </si>
+  <si>
+    <t>NEM US</t>
+  </si>
+  <si>
+    <t>纽曼矿业</t>
   </si>
   <si>
     <t>黄金</t>
   </si>
   <si>
-    <t>2382 HK</t>
-  </si>
-  <si>
-    <t>舜宇光学</t>
-  </si>
-  <si>
-    <t>光学/AI硬件</t>
-  </si>
-  <si>
-    <t>1024 HK</t>
-  </si>
-  <si>
-    <t>快手-W</t>
-  </si>
-  <si>
-    <t>互联网内容与信息</t>
-  </si>
-  <si>
-    <t>9988 HK</t>
-  </si>
-  <si>
-    <t>阿里巴巴</t>
-  </si>
-  <si>
-    <t>电商/云</t>
-  </si>
-  <si>
-    <t>20 HK</t>
-  </si>
-  <si>
-    <t>商汤-W</t>
+    <t>CRM US</t>
+  </si>
+  <si>
+    <t>赛富时</t>
   </si>
   <si>
     <t>应用软件</t>
   </si>
   <si>
-    <t>美股</t>
-  </si>
-  <si>
-    <t>ANET US</t>
-  </si>
-  <si>
-    <t>阿里斯塔</t>
-  </si>
-  <si>
-    <t>AI网络</t>
+    <t>META US</t>
+  </si>
+  <si>
+    <t>Meta平台</t>
+  </si>
+  <si>
+    <t>广告/AI</t>
+  </si>
+  <si>
+    <t>DASH US</t>
+  </si>
+  <si>
+    <t>DoorDash</t>
+  </si>
+  <si>
+    <t>互联网零售</t>
+  </si>
+  <si>
+    <t>WDAY US</t>
+  </si>
+  <si>
+    <t>Workday</t>
+  </si>
+  <si>
+    <t>MELI US</t>
+  </si>
+  <si>
+    <t>美客多</t>
   </si>
   <si>
     <t>APH US</t>
@@ -130,34 +191,43 @@
     <t>电子元件</t>
   </si>
   <si>
-    <t>NEM US</t>
-  </si>
-  <si>
-    <t>纽曼矿业</t>
-  </si>
-  <si>
-    <t>CRM US</t>
-  </si>
-  <si>
-    <t>赛富时</t>
-  </si>
-  <si>
-    <t>META US</t>
-  </si>
-  <si>
-    <t>Meta平台</t>
-  </si>
-  <si>
-    <t>广告/AI</t>
-  </si>
-  <si>
-    <t>MELI US</t>
-  </si>
-  <si>
-    <t>美客多</t>
-  </si>
-  <si>
-    <t>互联网零售</t>
+    <t>SPOT US</t>
+  </si>
+  <si>
+    <t>声田</t>
+  </si>
+  <si>
+    <t>MPWR US</t>
+  </si>
+  <si>
+    <t>芯源系统</t>
+  </si>
+  <si>
+    <t>半导体</t>
+  </si>
+  <si>
+    <t>GEV US</t>
+  </si>
+  <si>
+    <t>GE Vernova</t>
+  </si>
+  <si>
+    <t>专用工业机械</t>
+  </si>
+  <si>
+    <t>ASML US</t>
+  </si>
+  <si>
+    <t>阿斯麦</t>
+  </si>
+  <si>
+    <t>半导体设备</t>
+  </si>
+  <si>
+    <t>INTU US</t>
+  </si>
+  <si>
+    <t>财捷</t>
   </si>
   <si>
     <t>NU US</t>
@@ -167,57 +237,6 @@
   </si>
   <si>
     <t>区域性银行</t>
-  </si>
-  <si>
-    <t>WDAY US</t>
-  </si>
-  <si>
-    <t>Workday</t>
-  </si>
-  <si>
-    <t>SPOT US</t>
-  </si>
-  <si>
-    <t>声田</t>
-  </si>
-  <si>
-    <t>INTU US</t>
-  </si>
-  <si>
-    <t>财捷</t>
-  </si>
-  <si>
-    <t>GEV US</t>
-  </si>
-  <si>
-    <t>GE Vernova</t>
-  </si>
-  <si>
-    <t>专用工业机械</t>
-  </si>
-  <si>
-    <t>DASH US</t>
-  </si>
-  <si>
-    <t>DoorDash</t>
-  </si>
-  <si>
-    <t>MPWR US</t>
-  </si>
-  <si>
-    <t>芯源系统</t>
-  </si>
-  <si>
-    <t>半导体</t>
-  </si>
-  <si>
-    <t>ACN US</t>
-  </si>
-  <si>
-    <t>埃森哲</t>
-  </si>
-  <si>
-    <t>IT服务</t>
   </si>
 </sst>
 </file>
@@ -565,10 +584,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -597,7 +616,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -611,10 +630,10 @@
         <v>12</v>
       </c>
       <c r="E2">
-        <v>0.83</v>
+        <v>0.79</v>
       </c>
       <c r="F2">
-        <v>0.73</v>
+        <v>0.69</v>
       </c>
       <c r="G2" t="s">
         <v>13</v>
@@ -623,10 +642,18 @@
         <v>1.01</v>
       </c>
       <c r="I2" s="1">
-        <v>0.16300000000000001</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.15">
+        <v>0.14599999999999999</v>
+      </c>
+      <c r="K2">
+        <f>E2*100</f>
+        <v>79</v>
+      </c>
+      <c r="L2">
+        <f>F2*100</f>
+        <v>69</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -640,10 +667,10 @@
         <v>16</v>
       </c>
       <c r="E3">
-        <v>0.82</v>
+        <v>0.79</v>
       </c>
       <c r="F3">
-        <v>0.72</v>
+        <v>0.69</v>
       </c>
       <c r="G3" t="s">
         <v>13</v>
@@ -652,10 +679,18 @@
         <v>1.01</v>
       </c>
       <c r="I3" s="1">
-        <v>0.15160000000000001</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.15">
+        <v>0.13789999999999999</v>
+      </c>
+      <c r="K3">
+        <f>E3*100</f>
+        <v>79</v>
+      </c>
+      <c r="L3">
+        <f>F3*100</f>
+        <v>69</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -669,10 +704,10 @@
         <v>19</v>
       </c>
       <c r="E4">
-        <v>0.81</v>
+        <v>0.82</v>
       </c>
       <c r="F4">
-        <v>0.71</v>
+        <v>0.72</v>
       </c>
       <c r="G4" t="s">
         <v>13</v>
@@ -681,10 +716,18 @@
         <v>1.01</v>
       </c>
       <c r="I4" s="1">
-        <v>0.15279999999999999</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.15">
+        <v>0.15240000000000001</v>
+      </c>
+      <c r="K4">
+        <f>E4*100</f>
+        <v>82</v>
+      </c>
+      <c r="L4">
+        <f>F4*100</f>
+        <v>72</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -698,10 +741,10 @@
         <v>22</v>
       </c>
       <c r="E5">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="F5">
-        <v>0.72</v>
+        <v>0.75</v>
       </c>
       <c r="G5" t="s">
         <v>13</v>
@@ -710,10 +753,18 @@
         <v>1.01</v>
       </c>
       <c r="I5" s="1">
-        <v>0.14979999999999999</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.15">
+        <v>0.1469</v>
+      </c>
+      <c r="K5">
+        <f>E5*100</f>
+        <v>85</v>
+      </c>
+      <c r="L5">
+        <f>F5*100</f>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -727,10 +778,10 @@
         <v>25</v>
       </c>
       <c r="E6">
-        <v>0.85</v>
+        <v>0.82</v>
       </c>
       <c r="F6">
-        <v>0.75</v>
+        <v>0.72</v>
       </c>
       <c r="G6" t="s">
         <v>13</v>
@@ -739,10 +790,18 @@
         <v>1.01</v>
       </c>
       <c r="I6" s="1">
-        <v>0.14030000000000001</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.15">
+        <v>0.15390000000000001</v>
+      </c>
+      <c r="K6">
+        <f>E6*100</f>
+        <v>82</v>
+      </c>
+      <c r="L6">
+        <f>F6*100</f>
+        <v>72</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -756,10 +815,10 @@
         <v>28</v>
       </c>
       <c r="E7">
-        <v>0.84</v>
+        <v>0.85</v>
       </c>
       <c r="F7">
-        <v>0.74</v>
+        <v>0.75</v>
       </c>
       <c r="G7" t="s">
         <v>13</v>
@@ -768,10 +827,18 @@
         <v>1.01</v>
       </c>
       <c r="I7" s="1">
-        <v>0.21010000000000001</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.15">
+        <v>0.15609999999999999</v>
+      </c>
+      <c r="K7">
+        <f>E7*100</f>
+        <v>85</v>
+      </c>
+      <c r="L7">
+        <f>F7*100</f>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A8" t="s">
         <v>29</v>
       </c>
@@ -785,10 +852,10 @@
         <v>32</v>
       </c>
       <c r="E8">
-        <v>0.81</v>
+        <v>0.82</v>
       </c>
       <c r="F8">
-        <v>0.71</v>
+        <v>0.72</v>
       </c>
       <c r="G8" t="s">
         <v>13</v>
@@ -797,10 +864,18 @@
         <v>1.01</v>
       </c>
       <c r="I8" s="1">
-        <v>0.1789</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.15">
+        <v>0.1812</v>
+      </c>
+      <c r="K8">
+        <f>E8*100</f>
+        <v>82</v>
+      </c>
+      <c r="L8">
+        <f>F8*100</f>
+        <v>72</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A9" t="s">
         <v>29</v>
       </c>
@@ -814,10 +889,10 @@
         <v>35</v>
       </c>
       <c r="E9">
-        <v>0.83</v>
+        <v>0.85</v>
       </c>
       <c r="F9">
-        <v>0.73</v>
+        <v>0.75</v>
       </c>
       <c r="G9" t="s">
         <v>13</v>
@@ -826,10 +901,18 @@
         <v>1.01</v>
       </c>
       <c r="I9" s="1">
-        <v>0.1434</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.15">
+        <v>0.1333</v>
+      </c>
+      <c r="K9">
+        <f>E9*100</f>
+        <v>85</v>
+      </c>
+      <c r="L9">
+        <f>F9*100</f>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A10" t="s">
         <v>29</v>
       </c>
@@ -840,13 +923,13 @@
         <v>37</v>
       </c>
       <c r="D10" t="s">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="E10">
-        <v>0.85</v>
+        <v>0.84</v>
       </c>
       <c r="F10">
-        <v>0.75</v>
+        <v>0.74</v>
       </c>
       <c r="G10" t="s">
         <v>13</v>
@@ -855,27 +938,35 @@
         <v>1.01</v>
       </c>
       <c r="I10" s="1">
-        <v>0.13780000000000001</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.15">
+        <v>0.1366</v>
+      </c>
+      <c r="K10">
+        <f>E10*100</f>
+        <v>84</v>
+      </c>
+      <c r="L10">
+        <f>F10*100</f>
+        <v>74</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A11" t="s">
         <v>29</v>
       </c>
       <c r="B11" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C11" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D11" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="E11">
-        <v>0.84</v>
+        <v>0.85</v>
       </c>
       <c r="F11">
-        <v>0.74</v>
+        <v>0.75</v>
       </c>
       <c r="G11" t="s">
         <v>13</v>
@@ -884,27 +975,35 @@
         <v>1.01</v>
       </c>
       <c r="I11" s="1">
-        <v>0.1454</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.15">
+        <v>0.13550000000000001</v>
+      </c>
+      <c r="K11">
+        <f>E11*100</f>
+        <v>85</v>
+      </c>
+      <c r="L11">
+        <f>F11*100</f>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A12" t="s">
         <v>29</v>
       </c>
       <c r="B12" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C12" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D12" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E12">
-        <v>0.85</v>
+        <v>0.81</v>
       </c>
       <c r="F12">
-        <v>0.75</v>
+        <v>0.71</v>
       </c>
       <c r="G12" t="s">
         <v>13</v>
@@ -913,21 +1012,29 @@
         <v>1.01</v>
       </c>
       <c r="I12" s="1">
-        <v>0.1331</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.15">
+        <v>0.14660000000000001</v>
+      </c>
+      <c r="K12">
+        <f>E12*100</f>
+        <v>81</v>
+      </c>
+      <c r="L12">
+        <f>F12*100</f>
+        <v>71</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A13" t="s">
         <v>29</v>
       </c>
       <c r="B13" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C13" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D13" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="E13">
         <v>0.85</v>
@@ -942,27 +1049,35 @@
         <v>1.01</v>
       </c>
       <c r="I13" s="1">
-        <v>0.124</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.15">
+        <v>0.15390000000000001</v>
+      </c>
+      <c r="K13">
+        <f>E13*100</f>
+        <v>85</v>
+      </c>
+      <c r="L13">
+        <f>F13*100</f>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A14" t="s">
         <v>29</v>
       </c>
       <c r="B14" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C14" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D14" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E14">
-        <v>0.83</v>
+        <v>0.85</v>
       </c>
       <c r="F14">
-        <v>0.73</v>
+        <v>0.75</v>
       </c>
       <c r="G14" t="s">
         <v>13</v>
@@ -971,10 +1086,18 @@
         <v>1.01</v>
       </c>
       <c r="I14" s="1">
-        <v>0.15040000000000001</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.15">
+        <v>0.128</v>
+      </c>
+      <c r="K14">
+        <f>E14*100</f>
+        <v>85</v>
+      </c>
+      <c r="L14">
+        <f>F14*100</f>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A15" t="s">
         <v>29</v>
       </c>
@@ -985,13 +1108,13 @@
         <v>50</v>
       </c>
       <c r="D15" t="s">
-        <v>28</v>
+        <v>51</v>
       </c>
       <c r="E15">
-        <v>0.82</v>
+        <v>0.81</v>
       </c>
       <c r="F15">
-        <v>0.72</v>
+        <v>0.71</v>
       </c>
       <c r="G15" t="s">
         <v>13</v>
@@ -1000,21 +1123,29 @@
         <v>1.01</v>
       </c>
       <c r="I15" s="1">
-        <v>0.14829999999999999</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.15">
+        <v>0.11899999999999999</v>
+      </c>
+      <c r="K15">
+        <f>E15*100</f>
+        <v>81</v>
+      </c>
+      <c r="L15">
+        <f>F15*100</f>
+        <v>71</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A16" t="s">
         <v>29</v>
       </c>
       <c r="B16" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C16" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D16" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="E16">
         <v>0.85</v>
@@ -1029,27 +1160,35 @@
         <v>1.01</v>
       </c>
       <c r="I16" s="1">
-        <v>0.1394</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.15">
+        <v>0.14630000000000001</v>
+      </c>
+      <c r="K16">
+        <f>E16*100</f>
+        <v>85</v>
+      </c>
+      <c r="L16">
+        <f>F16*100</f>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A17" t="s">
         <v>29</v>
       </c>
       <c r="B17" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C17" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D17" t="s">
-        <v>28</v>
+        <v>56</v>
       </c>
       <c r="E17">
-        <v>0.84</v>
+        <v>0.82</v>
       </c>
       <c r="F17">
-        <v>0.74</v>
+        <v>0.72</v>
       </c>
       <c r="G17" t="s">
         <v>13</v>
@@ -1058,21 +1197,29 @@
         <v>1.01</v>
       </c>
       <c r="I17" s="1">
-        <v>0.19520000000000001</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.15">
+        <v>0.18959999999999999</v>
+      </c>
+      <c r="K17">
+        <f>E17*100</f>
+        <v>82</v>
+      </c>
+      <c r="L17">
+        <f>F17*100</f>
+        <v>72</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A18" t="s">
         <v>29</v>
       </c>
       <c r="B18" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C18" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D18" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E18">
         <v>0.8</v>
@@ -1087,27 +1234,35 @@
         <v>1.01</v>
       </c>
       <c r="I18" s="1">
-        <v>0.1409</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.15">
+        <v>0.14549999999999999</v>
+      </c>
+      <c r="K18">
+        <f>E18*100</f>
+        <v>80</v>
+      </c>
+      <c r="L18">
+        <f>F18*100</f>
+        <v>70</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A19" t="s">
         <v>29</v>
       </c>
       <c r="B19" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C19" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D19" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="E19">
-        <v>0.81</v>
+        <v>0.84</v>
       </c>
       <c r="F19">
-        <v>0.71</v>
+        <v>0.74</v>
       </c>
       <c r="G19" t="s">
         <v>13</v>
@@ -1116,27 +1271,35 @@
         <v>1.01</v>
       </c>
       <c r="I19" s="1">
-        <v>0.14910000000000001</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.15">
+        <v>0.13270000000000001</v>
+      </c>
+      <c r="K19">
+        <f>E19*100</f>
+        <v>84</v>
+      </c>
+      <c r="L19">
+        <f>F19*100</f>
+        <v>74</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A20" t="s">
         <v>29</v>
       </c>
       <c r="B20" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C20" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="D20" t="s">
-        <v>62</v>
+        <v>38</v>
       </c>
       <c r="E20">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="F20">
-        <v>0.72</v>
+        <v>0.75</v>
       </c>
       <c r="G20" t="s">
         <v>13</v>
@@ -1145,27 +1308,35 @@
         <v>1.01</v>
       </c>
       <c r="I20" s="1">
-        <v>0.19400000000000001</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.15">
+        <v>0.19539999999999999</v>
+      </c>
+      <c r="K20">
+        <f>E20*100</f>
+        <v>85</v>
+      </c>
+      <c r="L20">
+        <f>F20*100</f>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A21" t="s">
         <v>29</v>
       </c>
       <c r="B21" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C21" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D21" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E21">
-        <v>0.8</v>
+        <v>0.84</v>
       </c>
       <c r="F21">
-        <v>0.7</v>
+        <v>0.74</v>
       </c>
       <c r="G21" t="s">
         <v>13</v>
@@ -1174,7 +1345,15 @@
         <v>1.01</v>
       </c>
       <c r="I21" s="1">
-        <v>0.15010000000000001</v>
+        <v>0.1479</v>
+      </c>
+      <c r="K21">
+        <f>E21*100</f>
+        <v>84</v>
+      </c>
+      <c r="L21">
+        <f>F21*100</f>
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
W40 2026 weekly update
- 本周标的+票息, 名称/行业自动中文, 热度榜3328交行(IV<30)替换为英特尔, 重生成 watchlist.json(53只, 无NaN)
- 财经日历刷新至W40(回顾耐用品订单转正/消费信心48.1; 预告核心PCE9/30·美光9/30·埃森哲10/1·非农10/2)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/低波精选组.xlsx
+++ b/低波精选组.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Y:\GopherHK\Fixed Income\结构化产品\HTML 生成\FCN_Watchlist_交接\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE1733EE-2FCB-4A10-A70A-D28DD1CCF502}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F90EE3BF-B45C-4957-BE45-62DC9C702177}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-340" yWindow="10690" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" r:id="rId1"/>
@@ -152,6 +152,15 @@
     <t>应用软件</t>
   </si>
   <si>
+    <t>VLO US</t>
+  </si>
+  <si>
+    <t>瓦莱罗能源</t>
+  </si>
+  <si>
+    <t>油气炼化与销售</t>
+  </si>
+  <si>
     <t>META US</t>
   </si>
   <si>
@@ -161,6 +170,36 @@
     <t>广告/AI</t>
   </si>
   <si>
+    <t>APH US</t>
+  </si>
+  <si>
+    <t>安费诺</t>
+  </si>
+  <si>
+    <t>电子元件</t>
+  </si>
+  <si>
+    <t>WDAY US</t>
+  </si>
+  <si>
+    <t>Workday</t>
+  </si>
+  <si>
+    <t>SPOT US</t>
+  </si>
+  <si>
+    <t>声田</t>
+  </si>
+  <si>
+    <t>ASML US</t>
+  </si>
+  <si>
+    <t>阿斯麦</t>
+  </si>
+  <si>
+    <t>半导体设备</t>
+  </si>
+  <si>
     <t>DASH US</t>
   </si>
   <si>
@@ -170,73 +209,34 @@
     <t>互联网零售</t>
   </si>
   <si>
-    <t>WDAY US</t>
-  </si>
-  <si>
-    <t>Workday</t>
-  </si>
-  <si>
-    <t>MELI US</t>
-  </si>
-  <si>
-    <t>美客多</t>
-  </si>
-  <si>
-    <t>APH US</t>
-  </si>
-  <si>
-    <t>安费诺</t>
-  </si>
-  <si>
-    <t>电子元件</t>
-  </si>
-  <si>
-    <t>SPOT US</t>
-  </si>
-  <si>
-    <t>声田</t>
-  </si>
-  <si>
-    <t>MPWR US</t>
-  </si>
-  <si>
-    <t>芯源系统</t>
+    <t>PWR US</t>
+  </si>
+  <si>
+    <t>广达服务</t>
+  </si>
+  <si>
+    <t>工程与建筑</t>
+  </si>
+  <si>
+    <t>MCHP US</t>
+  </si>
+  <si>
+    <t>微芯科技</t>
   </si>
   <si>
     <t>半导体</t>
   </si>
   <si>
-    <t>GEV US</t>
-  </si>
-  <si>
-    <t>GE Vernova</t>
-  </si>
-  <si>
-    <t>专用工业机械</t>
-  </si>
-  <si>
-    <t>ASML US</t>
-  </si>
-  <si>
-    <t>阿斯麦</t>
-  </si>
-  <si>
-    <t>半导体设备</t>
-  </si>
-  <si>
-    <t>INTU US</t>
-  </si>
-  <si>
-    <t>财捷</t>
-  </si>
-  <si>
-    <t>NU US</t>
-  </si>
-  <si>
-    <t>Nu控股</t>
-  </si>
-  <si>
-    <t>区域性银行</t>
+    <t>NXPI US</t>
+  </si>
+  <si>
+    <t>恩智浦</t>
+  </si>
+  <si>
+    <t>TXN US</t>
+  </si>
+  <si>
+    <t>德州仪器</t>
   </si>
 </sst>
 </file>
@@ -584,10 +584,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -616,7 +616,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -630,10 +630,10 @@
         <v>12</v>
       </c>
       <c r="E2">
-        <v>0.79</v>
+        <v>0.84</v>
       </c>
       <c r="F2">
-        <v>0.69</v>
+        <v>0.74</v>
       </c>
       <c r="G2" t="s">
         <v>13</v>
@@ -642,18 +642,10 @@
         <v>1.01</v>
       </c>
       <c r="I2" s="1">
-        <v>0.14599999999999999</v>
-      </c>
-      <c r="K2">
-        <f>E2*100</f>
-        <v>79</v>
-      </c>
-      <c r="L2">
-        <f>F2*100</f>
-        <v>69</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.15">
+        <v>0.18720000000000001</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -667,10 +659,10 @@
         <v>16</v>
       </c>
       <c r="E3">
-        <v>0.79</v>
+        <v>0.81</v>
       </c>
       <c r="F3">
-        <v>0.69</v>
+        <v>0.71</v>
       </c>
       <c r="G3" t="s">
         <v>13</v>
@@ -679,18 +671,10 @@
         <v>1.01</v>
       </c>
       <c r="I3" s="1">
-        <v>0.13789999999999999</v>
-      </c>
-      <c r="K3">
-        <f>E3*100</f>
-        <v>79</v>
-      </c>
-      <c r="L3">
-        <f>F3*100</f>
-        <v>69</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.15">
+        <v>0.1507</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -704,10 +688,10 @@
         <v>19</v>
       </c>
       <c r="E4">
-        <v>0.82</v>
+        <v>0.83</v>
       </c>
       <c r="F4">
-        <v>0.72</v>
+        <v>0.73</v>
       </c>
       <c r="G4" t="s">
         <v>13</v>
@@ -716,18 +700,10 @@
         <v>1.01</v>
       </c>
       <c r="I4" s="1">
-        <v>0.15240000000000001</v>
-      </c>
-      <c r="K4">
-        <f>E4*100</f>
-        <v>82</v>
-      </c>
-      <c r="L4">
-        <f>F4*100</f>
-        <v>72</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.15">
+        <v>0.1532</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -753,18 +729,10 @@
         <v>1.01</v>
       </c>
       <c r="I5" s="1">
-        <v>0.1469</v>
-      </c>
-      <c r="K5">
-        <f>E5*100</f>
-        <v>85</v>
-      </c>
-      <c r="L5">
-        <f>F5*100</f>
-        <v>75</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.15">
+        <v>0.13389999999999999</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -790,18 +758,10 @@
         <v>1.01</v>
       </c>
       <c r="I6" s="1">
-        <v>0.15390000000000001</v>
-      </c>
-      <c r="K6">
-        <f>E6*100</f>
-        <v>82</v>
-      </c>
-      <c r="L6">
-        <f>F6*100</f>
-        <v>72</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.15">
+        <v>0.1565</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -827,18 +787,10 @@
         <v>1.01</v>
       </c>
       <c r="I7" s="1">
-        <v>0.15609999999999999</v>
-      </c>
-      <c r="K7">
-        <f>E7*100</f>
-        <v>85</v>
-      </c>
-      <c r="L7">
-        <f>F7*100</f>
-        <v>75</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.15">
+        <v>0.15770000000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A8" t="s">
         <v>29</v>
       </c>
@@ -852,10 +804,10 @@
         <v>32</v>
       </c>
       <c r="E8">
-        <v>0.82</v>
+        <v>0.84</v>
       </c>
       <c r="F8">
-        <v>0.72</v>
+        <v>0.74</v>
       </c>
       <c r="G8" t="s">
         <v>13</v>
@@ -864,18 +816,10 @@
         <v>1.01</v>
       </c>
       <c r="I8" s="1">
-        <v>0.1812</v>
-      </c>
-      <c r="K8">
-        <f>E8*100</f>
-        <v>82</v>
-      </c>
-      <c r="L8">
-        <f>F8*100</f>
-        <v>72</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.15">
+        <v>0.2046</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A9" t="s">
         <v>29</v>
       </c>
@@ -901,18 +845,10 @@
         <v>1.01</v>
       </c>
       <c r="I9" s="1">
-        <v>0.1333</v>
-      </c>
-      <c r="K9">
-        <f>E9*100</f>
-        <v>85</v>
-      </c>
-      <c r="L9">
-        <f>F9*100</f>
-        <v>75</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.15">
+        <v>0.13750000000000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A10" t="s">
         <v>29</v>
       </c>
@@ -938,18 +874,10 @@
         <v>1.01</v>
       </c>
       <c r="I10" s="1">
-        <v>0.1366</v>
-      </c>
-      <c r="K10">
-        <f>E10*100</f>
-        <v>84</v>
-      </c>
-      <c r="L10">
-        <f>F10*100</f>
-        <v>74</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.15">
+        <v>0.1391</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A11" t="s">
         <v>29</v>
       </c>
@@ -963,10 +891,10 @@
         <v>41</v>
       </c>
       <c r="E11">
-        <v>0.85</v>
+        <v>0.84</v>
       </c>
       <c r="F11">
-        <v>0.75</v>
+        <v>0.74</v>
       </c>
       <c r="G11" t="s">
         <v>13</v>
@@ -975,18 +903,10 @@
         <v>1.01</v>
       </c>
       <c r="I11" s="1">
-        <v>0.13550000000000001</v>
-      </c>
-      <c r="K11">
-        <f>E11*100</f>
-        <v>85</v>
-      </c>
-      <c r="L11">
-        <f>F11*100</f>
-        <v>75</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.15">
+        <v>0.19869999999999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A12" t="s">
         <v>29</v>
       </c>
@@ -1000,10 +920,10 @@
         <v>44</v>
       </c>
       <c r="E12">
-        <v>0.81</v>
+        <v>0.85</v>
       </c>
       <c r="F12">
-        <v>0.71</v>
+        <v>0.75</v>
       </c>
       <c r="G12" t="s">
         <v>13</v>
@@ -1012,18 +932,10 @@
         <v>1.01</v>
       </c>
       <c r="I12" s="1">
-        <v>0.14660000000000001</v>
-      </c>
-      <c r="K12">
-        <f>E12*100</f>
-        <v>81</v>
-      </c>
-      <c r="L12">
-        <f>F12*100</f>
-        <v>71</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.15">
+        <v>0.13980000000000001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A13" t="s">
         <v>29</v>
       </c>
@@ -1034,88 +946,72 @@
         <v>46</v>
       </c>
       <c r="D13" t="s">
+        <v>47</v>
+      </c>
+      <c r="E13">
+        <v>0.84</v>
+      </c>
+      <c r="F13">
+        <v>0.74</v>
+      </c>
+      <c r="G13" t="s">
+        <v>13</v>
+      </c>
+      <c r="H13">
+        <v>1.01</v>
+      </c>
+      <c r="I13" s="1">
+        <v>0.13880000000000001</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.15">
+      <c r="A14" t="s">
+        <v>29</v>
+      </c>
+      <c r="B14" t="s">
+        <v>48</v>
+      </c>
+      <c r="C14" t="s">
+        <v>49</v>
+      </c>
+      <c r="D14" t="s">
         <v>38</v>
       </c>
-      <c r="E13">
+      <c r="E14">
+        <v>0.82</v>
+      </c>
+      <c r="F14">
+        <v>0.72</v>
+      </c>
+      <c r="G14" t="s">
+        <v>13</v>
+      </c>
+      <c r="H14">
+        <v>1.01</v>
+      </c>
+      <c r="I14" s="1">
+        <v>0.1474</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.15">
+      <c r="A15" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" t="s">
+        <v>50</v>
+      </c>
+      <c r="C15" t="s">
+        <v>51</v>
+      </c>
+      <c r="D15" t="s">
+        <v>25</v>
+      </c>
+      <c r="E15">
         <v>0.85</v>
       </c>
-      <c r="F13">
+      <c r="F15">
         <v>0.75</v>
       </c>
-      <c r="G13" t="s">
-        <v>13</v>
-      </c>
-      <c r="H13">
-        <v>1.01</v>
-      </c>
-      <c r="I13" s="1">
-        <v>0.15390000000000001</v>
-      </c>
-      <c r="K13">
-        <f>E13*100</f>
-        <v>85</v>
-      </c>
-      <c r="L13">
-        <f>F13*100</f>
-        <v>75</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.15">
-      <c r="A14" t="s">
-        <v>29</v>
-      </c>
-      <c r="B14" t="s">
-        <v>47</v>
-      </c>
-      <c r="C14" t="s">
-        <v>48</v>
-      </c>
-      <c r="D14" t="s">
-        <v>44</v>
-      </c>
-      <c r="E14">
-        <v>0.85</v>
-      </c>
-      <c r="F14">
-        <v>0.75</v>
-      </c>
-      <c r="G14" t="s">
-        <v>13</v>
-      </c>
-      <c r="H14">
-        <v>1.01</v>
-      </c>
-      <c r="I14" s="1">
-        <v>0.128</v>
-      </c>
-      <c r="K14">
-        <f>E14*100</f>
-        <v>85</v>
-      </c>
-      <c r="L14">
-        <f>F14*100</f>
-        <v>75</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.15">
-      <c r="A15" t="s">
-        <v>29</v>
-      </c>
-      <c r="B15" t="s">
-        <v>49</v>
-      </c>
-      <c r="C15" t="s">
-        <v>50</v>
-      </c>
-      <c r="D15" t="s">
-        <v>51</v>
-      </c>
-      <c r="E15">
-        <v>0.81</v>
-      </c>
-      <c r="F15">
-        <v>0.71</v>
-      </c>
       <c r="G15" t="s">
         <v>13</v>
       </c>
@@ -1123,18 +1019,10 @@
         <v>1.01</v>
       </c>
       <c r="I15" s="1">
-        <v>0.11899999999999999</v>
-      </c>
-      <c r="K15">
-        <f>E15*100</f>
-        <v>81</v>
-      </c>
-      <c r="L15">
-        <f>F15*100</f>
-        <v>71</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.15">
+        <v>0.161</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A16" t="s">
         <v>29</v>
       </c>
@@ -1145,7 +1033,7 @@
         <v>53</v>
       </c>
       <c r="D16" t="s">
-        <v>25</v>
+        <v>54</v>
       </c>
       <c r="E16">
         <v>0.85</v>
@@ -1160,35 +1048,27 @@
         <v>1.01</v>
       </c>
       <c r="I16" s="1">
-        <v>0.14630000000000001</v>
-      </c>
-      <c r="K16">
-        <f>E16*100</f>
-        <v>85</v>
-      </c>
-      <c r="L16">
-        <f>F16*100</f>
-        <v>75</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.15">
+        <v>0.14660000000000001</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A17" t="s">
         <v>29</v>
       </c>
       <c r="B17" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C17" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D17" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E17">
-        <v>0.82</v>
+        <v>0.81</v>
       </c>
       <c r="F17">
-        <v>0.72</v>
+        <v>0.71</v>
       </c>
       <c r="G17" t="s">
         <v>13</v>
@@ -1197,35 +1077,27 @@
         <v>1.01</v>
       </c>
       <c r="I17" s="1">
-        <v>0.18959999999999999</v>
-      </c>
-      <c r="K17">
-        <f>E17*100</f>
-        <v>82</v>
-      </c>
-      <c r="L17">
-        <f>F17*100</f>
-        <v>72</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.15">
+        <v>0.15670000000000001</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A18" t="s">
         <v>29</v>
       </c>
       <c r="B18" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C18" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D18" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E18">
-        <v>0.8</v>
+        <v>0.84</v>
       </c>
       <c r="F18">
-        <v>0.7</v>
+        <v>0.74</v>
       </c>
       <c r="G18" t="s">
         <v>13</v>
@@ -1234,35 +1106,27 @@
         <v>1.01</v>
       </c>
       <c r="I18" s="1">
-        <v>0.14549999999999999</v>
-      </c>
-      <c r="K18">
-        <f>E18*100</f>
-        <v>80</v>
-      </c>
-      <c r="L18">
-        <f>F18*100</f>
-        <v>70</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.15">
+        <v>0.13139999999999999</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A19" t="s">
         <v>29</v>
       </c>
       <c r="B19" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C19" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D19" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E19">
-        <v>0.84</v>
+        <v>0.85</v>
       </c>
       <c r="F19">
-        <v>0.74</v>
+        <v>0.75</v>
       </c>
       <c r="G19" t="s">
         <v>13</v>
@@ -1271,73 +1135,57 @@
         <v>1.01</v>
       </c>
       <c r="I19" s="1">
-        <v>0.13270000000000001</v>
-      </c>
-      <c r="K19">
-        <f>E19*100</f>
-        <v>84</v>
-      </c>
-      <c r="L19">
-        <f>F19*100</f>
-        <v>74</v>
-      </c>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.15">
+        <v>0.21829999999999999</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A20" t="s">
         <v>29</v>
       </c>
       <c r="B20" t="s">
+        <v>64</v>
+      </c>
+      <c r="C20" t="s">
+        <v>65</v>
+      </c>
+      <c r="D20" t="s">
         <v>63</v>
       </c>
-      <c r="C20" t="s">
-        <v>64</v>
-      </c>
-      <c r="D20" t="s">
-        <v>38</v>
-      </c>
       <c r="E20">
+        <v>0.81</v>
+      </c>
+      <c r="F20">
+        <v>0.71</v>
+      </c>
+      <c r="G20" t="s">
+        <v>13</v>
+      </c>
+      <c r="H20">
+        <v>1.01</v>
+      </c>
+      <c r="I20" s="1">
+        <v>0.1467</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.15">
+      <c r="A21" t="s">
+        <v>29</v>
+      </c>
+      <c r="B21" t="s">
+        <v>66</v>
+      </c>
+      <c r="C21" t="s">
+        <v>67</v>
+      </c>
+      <c r="D21" t="s">
+        <v>63</v>
+      </c>
+      <c r="E21">
         <v>0.85</v>
       </c>
-      <c r="F20">
+      <c r="F21">
         <v>0.75</v>
       </c>
-      <c r="G20" t="s">
-        <v>13</v>
-      </c>
-      <c r="H20">
-        <v>1.01</v>
-      </c>
-      <c r="I20" s="1">
-        <v>0.19539999999999999</v>
-      </c>
-      <c r="K20">
-        <f>E20*100</f>
-        <v>85</v>
-      </c>
-      <c r="L20">
-        <f>F20*100</f>
-        <v>75</v>
-      </c>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.15">
-      <c r="A21" t="s">
-        <v>29</v>
-      </c>
-      <c r="B21" t="s">
-        <v>65</v>
-      </c>
-      <c r="C21" t="s">
-        <v>66</v>
-      </c>
-      <c r="D21" t="s">
-        <v>67</v>
-      </c>
-      <c r="E21">
-        <v>0.84</v>
-      </c>
-      <c r="F21">
-        <v>0.74</v>
-      </c>
       <c r="G21" t="s">
         <v>13</v>
       </c>
@@ -1345,15 +1193,7 @@
         <v>1.01</v>
       </c>
       <c r="I21" s="1">
-        <v>0.1479</v>
-      </c>
-      <c r="K21">
-        <f>E21*100</f>
-        <v>84</v>
-      </c>
-      <c r="L21">
-        <f>F21*100</f>
-        <v>74</v>
+        <v>0.1545</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
W41 2026 weekly update
- 本周标的+票息, 名称/行业自动中文, 重生成 watchlist.json(53只)
- 修复: generate _validate_ana/出表对DeepSeek偶返回list的防护(此前崩溃致未写出)
- 财经日历刷新至W41(回顾核心PCE降温至3.0%/美光创纪录/10月政府停摆致数据推迟; 预告停摆数据空窗·Q3财报季·阿斯麦10/15)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/低波精选组.xlsx
+++ b/低波精选组.xlsx
@@ -8,27 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Y:\GopherHK\Fixed Income\结构化产品\HTML 生成\FCN_Watchlist_交接\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F90EE3BF-B45C-4957-BE45-62DC9C702177}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE42B250-F594-421D-9D21-A8A435EE3827}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-340" yWindow="10690" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -95,6 +82,15 @@
     <t>光学/AI硬件</t>
   </si>
   <si>
+    <t>1024 HK</t>
+  </si>
+  <si>
+    <t>快手-W</t>
+  </si>
+  <si>
+    <t>互联网内容与信息</t>
+  </si>
+  <si>
     <t>9988 HK</t>
   </si>
   <si>
@@ -104,27 +100,27 @@
     <t>电商/云</t>
   </si>
   <si>
-    <t>1024 HK</t>
-  </si>
-  <si>
-    <t>快手-W</t>
-  </si>
-  <si>
-    <t>互联网内容与信息</t>
-  </si>
-  <si>
-    <t>1810 HK</t>
-  </si>
-  <si>
-    <t>小米集团</t>
-  </si>
-  <si>
-    <t>AI/IoT</t>
+    <t>20 HK</t>
+  </si>
+  <si>
+    <t>商汤-W</t>
+  </si>
+  <si>
+    <t>应用软件</t>
   </si>
   <si>
     <t>美股</t>
   </si>
   <si>
+    <t>AMD US</t>
+  </si>
+  <si>
+    <t>超微半导体</t>
+  </si>
+  <si>
+    <t>AI芯片</t>
+  </si>
+  <si>
     <t>ANET US</t>
   </si>
   <si>
@@ -134,6 +130,39 @@
     <t>AI网络</t>
   </si>
   <si>
+    <t>PLTR US</t>
+  </si>
+  <si>
+    <t>帕兰提尔</t>
+  </si>
+  <si>
+    <t>AI软件</t>
+  </si>
+  <si>
+    <t>APH US</t>
+  </si>
+  <si>
+    <t>安费诺</t>
+  </si>
+  <si>
+    <t>电子元件</t>
+  </si>
+  <si>
+    <t>CRM US</t>
+  </si>
+  <si>
+    <t>赛富时</t>
+  </si>
+  <si>
+    <t>VLO US</t>
+  </si>
+  <si>
+    <t>瓦莱罗能源</t>
+  </si>
+  <si>
+    <t>油气炼化与销售</t>
+  </si>
+  <si>
     <t>NEM US</t>
   </si>
   <si>
@@ -143,22 +172,10 @@
     <t>黄金</t>
   </si>
   <si>
-    <t>CRM US</t>
-  </si>
-  <si>
-    <t>赛富时</t>
-  </si>
-  <si>
-    <t>应用软件</t>
-  </si>
-  <si>
-    <t>VLO US</t>
-  </si>
-  <si>
-    <t>瓦莱罗能源</t>
-  </si>
-  <si>
-    <t>油气炼化与销售</t>
+    <t>NOW US</t>
+  </si>
+  <si>
+    <t>ServiceNow</t>
   </si>
   <si>
     <t>META US</t>
@@ -170,13 +187,22 @@
     <t>广告/AI</t>
   </si>
   <si>
-    <t>APH US</t>
-  </si>
-  <si>
-    <t>安费诺</t>
-  </si>
-  <si>
-    <t>电子元件</t>
+    <t>ASML US</t>
+  </si>
+  <si>
+    <t>阿斯麦</t>
+  </si>
+  <si>
+    <t>半导体设备</t>
+  </si>
+  <si>
+    <t>PWR US</t>
+  </si>
+  <si>
+    <t>广达服务</t>
+  </si>
+  <si>
+    <t>工程与建筑</t>
   </si>
   <si>
     <t>WDAY US</t>
@@ -185,39 +211,6 @@
     <t>Workday</t>
   </si>
   <si>
-    <t>SPOT US</t>
-  </si>
-  <si>
-    <t>声田</t>
-  </si>
-  <si>
-    <t>ASML US</t>
-  </si>
-  <si>
-    <t>阿斯麦</t>
-  </si>
-  <si>
-    <t>半导体设备</t>
-  </si>
-  <si>
-    <t>DASH US</t>
-  </si>
-  <si>
-    <t>DoorDash</t>
-  </si>
-  <si>
-    <t>互联网零售</t>
-  </si>
-  <si>
-    <t>PWR US</t>
-  </si>
-  <si>
-    <t>广达服务</t>
-  </si>
-  <si>
-    <t>工程与建筑</t>
-  </si>
-  <si>
     <t>MCHP US</t>
   </si>
   <si>
@@ -231,12 +224,6 @@
   </si>
   <si>
     <t>恩智浦</t>
-  </si>
-  <si>
-    <t>TXN US</t>
-  </si>
-  <si>
-    <t>德州仪器</t>
   </si>
 </sst>
 </file>
@@ -586,6 +573,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I21"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
+  <cols>
+    <col min="9" max="9" width="9.5" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A1" t="s">
@@ -630,10 +620,10 @@
         <v>12</v>
       </c>
       <c r="E2">
-        <v>0.84</v>
+        <v>0.8</v>
       </c>
       <c r="F2">
-        <v>0.74</v>
+        <v>0.7</v>
       </c>
       <c r="G2" t="s">
         <v>13</v>
@@ -642,7 +632,7 @@
         <v>1.01</v>
       </c>
       <c r="I2" s="1">
-        <v>0.18720000000000001</v>
+        <v>0.16120000000000001</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.15">
@@ -671,7 +661,7 @@
         <v>1.01</v>
       </c>
       <c r="I3" s="1">
-        <v>0.1507</v>
+        <v>0.15970000000000001</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.15">
@@ -688,10 +678,10 @@
         <v>19</v>
       </c>
       <c r="E4">
-        <v>0.83</v>
+        <v>0.84</v>
       </c>
       <c r="F4">
-        <v>0.73</v>
+        <v>0.74</v>
       </c>
       <c r="G4" t="s">
         <v>13</v>
@@ -700,7 +690,7 @@
         <v>1.01</v>
       </c>
       <c r="I4" s="1">
-        <v>0.1532</v>
+        <v>0.14879999999999999</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.15">
@@ -717,10 +707,10 @@
         <v>22</v>
       </c>
       <c r="E5">
-        <v>0.85</v>
+        <v>0.82</v>
       </c>
       <c r="F5">
-        <v>0.75</v>
+        <v>0.72</v>
       </c>
       <c r="G5" t="s">
         <v>13</v>
@@ -729,7 +719,7 @@
         <v>1.01</v>
       </c>
       <c r="I5" s="1">
-        <v>0.13389999999999999</v>
+        <v>0.15429999999999999</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.15">
@@ -746,10 +736,10 @@
         <v>25</v>
       </c>
       <c r="E6">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="F6">
-        <v>0.72</v>
+        <v>0.75</v>
       </c>
       <c r="G6" t="s">
         <v>13</v>
@@ -758,7 +748,7 @@
         <v>1.01</v>
       </c>
       <c r="I6" s="1">
-        <v>0.1565</v>
+        <v>0.122</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.15">
@@ -775,10 +765,10 @@
         <v>28</v>
       </c>
       <c r="E7">
-        <v>0.85</v>
+        <v>0.79</v>
       </c>
       <c r="F7">
-        <v>0.75</v>
+        <v>0.69</v>
       </c>
       <c r="G7" t="s">
         <v>13</v>
@@ -787,7 +777,7 @@
         <v>1.01</v>
       </c>
       <c r="I7" s="1">
-        <v>0.15770000000000001</v>
+        <v>0.1535</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.15">
@@ -804,10 +794,10 @@
         <v>32</v>
       </c>
       <c r="E8">
-        <v>0.84</v>
+        <v>0.83</v>
       </c>
       <c r="F8">
-        <v>0.74</v>
+        <v>0.73</v>
       </c>
       <c r="G8" t="s">
         <v>13</v>
@@ -816,7 +806,7 @@
         <v>1.01</v>
       </c>
       <c r="I8" s="1">
-        <v>0.2046</v>
+        <v>0.19489999999999999</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.15">
@@ -833,10 +823,10 @@
         <v>35</v>
       </c>
       <c r="E9">
-        <v>0.85</v>
+        <v>0.83</v>
       </c>
       <c r="F9">
-        <v>0.75</v>
+        <v>0.73</v>
       </c>
       <c r="G9" t="s">
         <v>13</v>
@@ -845,7 +835,7 @@
         <v>1.01</v>
       </c>
       <c r="I9" s="1">
-        <v>0.13750000000000001</v>
+        <v>0.19520000000000001</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.15">
@@ -862,10 +852,10 @@
         <v>38</v>
       </c>
       <c r="E10">
-        <v>0.84</v>
+        <v>0.82</v>
       </c>
       <c r="F10">
-        <v>0.74</v>
+        <v>0.72</v>
       </c>
       <c r="G10" t="s">
         <v>13</v>
@@ -874,7 +864,7 @@
         <v>1.01</v>
       </c>
       <c r="I10" s="1">
-        <v>0.1391</v>
+        <v>0.20749999999999999</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.15">
@@ -903,7 +893,7 @@
         <v>1.01</v>
       </c>
       <c r="I11" s="1">
-        <v>0.19869999999999999</v>
+        <v>0.14419999999999999</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.15">
@@ -917,13 +907,13 @@
         <v>43</v>
       </c>
       <c r="D12" t="s">
-        <v>44</v>
+        <v>28</v>
       </c>
       <c r="E12">
-        <v>0.85</v>
+        <v>0.84</v>
       </c>
       <c r="F12">
-        <v>0.75</v>
+        <v>0.74</v>
       </c>
       <c r="G12" t="s">
         <v>13</v>
@@ -932,7 +922,7 @@
         <v>1.01</v>
       </c>
       <c r="I12" s="1">
-        <v>0.13980000000000001</v>
+        <v>0.14410000000000001</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.15">
@@ -940,19 +930,19 @@
         <v>29</v>
       </c>
       <c r="B13" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13" t="s">
         <v>45</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>46</v>
       </c>
-      <c r="D13" t="s">
-        <v>47</v>
-      </c>
       <c r="E13">
-        <v>0.84</v>
+        <v>0.79</v>
       </c>
       <c r="F13">
-        <v>0.74</v>
+        <v>0.69</v>
       </c>
       <c r="G13" t="s">
         <v>13</v>
@@ -961,7 +951,7 @@
         <v>1.01</v>
       </c>
       <c r="I13" s="1">
-        <v>0.13880000000000001</v>
+        <v>0.14799999999999999</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.15">
@@ -969,19 +959,19 @@
         <v>29</v>
       </c>
       <c r="B14" t="s">
+        <v>47</v>
+      </c>
+      <c r="C14" t="s">
         <v>48</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>49</v>
       </c>
-      <c r="D14" t="s">
-        <v>38</v>
-      </c>
       <c r="E14">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="F14">
-        <v>0.72</v>
+        <v>0.75</v>
       </c>
       <c r="G14" t="s">
         <v>13</v>
@@ -990,7 +980,7 @@
         <v>1.01</v>
       </c>
       <c r="I14" s="1">
-        <v>0.1474</v>
+        <v>0.1249</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.15">
@@ -1004,13 +994,13 @@
         <v>51</v>
       </c>
       <c r="D15" t="s">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="E15">
-        <v>0.85</v>
+        <v>0.83</v>
       </c>
       <c r="F15">
-        <v>0.75</v>
+        <v>0.73</v>
       </c>
       <c r="G15" t="s">
         <v>13</v>
@@ -1019,7 +1009,7 @@
         <v>1.01</v>
       </c>
       <c r="I15" s="1">
-        <v>0.161</v>
+        <v>0.20180000000000001</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.15">
@@ -1048,7 +1038,7 @@
         <v>1.01</v>
       </c>
       <c r="I16" s="1">
-        <v>0.14660000000000001</v>
+        <v>0.12130000000000001</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.15">
@@ -1065,10 +1055,10 @@
         <v>57</v>
       </c>
       <c r="E17">
-        <v>0.81</v>
+        <v>0.84</v>
       </c>
       <c r="F17">
-        <v>0.71</v>
+        <v>0.74</v>
       </c>
       <c r="G17" t="s">
         <v>13</v>
@@ -1077,7 +1067,7 @@
         <v>1.01</v>
       </c>
       <c r="I17" s="1">
-        <v>0.15670000000000001</v>
+        <v>0.13919999999999999</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.15">
@@ -1094,10 +1084,10 @@
         <v>60</v>
       </c>
       <c r="E18">
-        <v>0.84</v>
+        <v>0.85</v>
       </c>
       <c r="F18">
-        <v>0.74</v>
+        <v>0.75</v>
       </c>
       <c r="G18" t="s">
         <v>13</v>
@@ -1106,7 +1096,7 @@
         <v>1.01</v>
       </c>
       <c r="I18" s="1">
-        <v>0.13139999999999999</v>
+        <v>0.13880000000000001</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.15">
@@ -1120,13 +1110,13 @@
         <v>62</v>
       </c>
       <c r="D19" t="s">
-        <v>63</v>
+        <v>28</v>
       </c>
       <c r="E19">
-        <v>0.85</v>
+        <v>0.81</v>
       </c>
       <c r="F19">
-        <v>0.75</v>
+        <v>0.71</v>
       </c>
       <c r="G19" t="s">
         <v>13</v>
@@ -1135,7 +1125,7 @@
         <v>1.01</v>
       </c>
       <c r="I19" s="1">
-        <v>0.21829999999999999</v>
+        <v>0.14180000000000001</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.15">
@@ -1143,19 +1133,19 @@
         <v>29</v>
       </c>
       <c r="B20" t="s">
+        <v>63</v>
+      </c>
+      <c r="C20" t="s">
         <v>64</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
         <v>65</v>
       </c>
-      <c r="D20" t="s">
-        <v>63</v>
-      </c>
       <c r="E20">
-        <v>0.81</v>
+        <v>0.85</v>
       </c>
       <c r="F20">
-        <v>0.71</v>
+        <v>0.75</v>
       </c>
       <c r="G20" t="s">
         <v>13</v>
@@ -1164,7 +1154,7 @@
         <v>1.01</v>
       </c>
       <c r="I20" s="1">
-        <v>0.1467</v>
+        <v>0.21440000000000001</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.15">
@@ -1178,13 +1168,13 @@
         <v>67</v>
       </c>
       <c r="D21" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E21">
-        <v>0.85</v>
+        <v>0.83</v>
       </c>
       <c r="F21">
-        <v>0.75</v>
+        <v>0.73</v>
       </c>
       <c r="G21" t="s">
         <v>13</v>
@@ -1193,7 +1183,7 @@
         <v>1.01</v>
       </c>
       <c r="I21" s="1">
-        <v>0.1545</v>
+        <v>0.14899999999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
W42 2026 weekly update
- 本周标的+票息, 名称/行业自动中文, 重生成 watchlist.json(51只)
- 财经日历刷新至W42(回顾FOMC纪要确认9月加息至3.75-4.00%; 预告Q3财报季·阿斯麦10/14·台积电10/15·奈飞10/20·下次议息10/28)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/低波精选组.xlsx
+++ b/低波精选组.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Y:\GopherHK\Fixed Income\结构化产品\HTML 生成\FCN_Watchlist_交接\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE42B250-F594-421D-9D21-A8A435EE3827}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29877FFB-46A7-4FE9-AE4B-FC95954F0F04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" r:id="rId1"/>
@@ -52,25 +52,25 @@
     <t>港股</t>
   </si>
   <si>
-    <t>1093 HK</t>
-  </si>
-  <si>
-    <t>石药集团</t>
-  </si>
-  <si>
-    <t>制药</t>
+    <t>2359 HK</t>
+  </si>
+  <si>
+    <t>药明康德</t>
+  </si>
+  <si>
+    <t>诊断与研究</t>
   </si>
   <si>
     <t>欧式敲入</t>
   </si>
   <si>
-    <t>2359 HK</t>
-  </si>
-  <si>
-    <t>药明康德</t>
-  </si>
-  <si>
-    <t>诊断与研究</t>
+    <t>2269 HK</t>
+  </si>
+  <si>
+    <t>药明生物</t>
+  </si>
+  <si>
+    <t>生物科技</t>
   </si>
   <si>
     <t>2382 HK</t>
@@ -154,6 +154,15 @@
     <t>赛富时</t>
   </si>
   <si>
+    <t>NU US</t>
+  </si>
+  <si>
+    <t>Nu控股</t>
+  </si>
+  <si>
+    <t>区域性银行</t>
+  </si>
+  <si>
     <t>VLO US</t>
   </si>
   <si>
@@ -163,6 +172,12 @@
     <t>油气炼化与销售</t>
   </si>
   <si>
+    <t>NOW US</t>
+  </si>
+  <si>
+    <t>ServiceNow</t>
+  </si>
+  <si>
     <t>NEM US</t>
   </si>
   <si>
@@ -172,19 +187,25 @@
     <t>黄金</t>
   </si>
   <si>
-    <t>NOW US</t>
-  </si>
-  <si>
-    <t>ServiceNow</t>
-  </si>
-  <si>
-    <t>META US</t>
-  </si>
-  <si>
-    <t>Meta平台</t>
-  </si>
-  <si>
-    <t>广告/AI</t>
+    <t>SPOT US</t>
+  </si>
+  <si>
+    <t>声田</t>
+  </si>
+  <si>
+    <t>AMAT US</t>
+  </si>
+  <si>
+    <t>应用材料</t>
+  </si>
+  <si>
+    <t>半导体设备与材料</t>
+  </si>
+  <si>
+    <t>WDAY US</t>
+  </si>
+  <si>
+    <t>Workday</t>
   </si>
   <si>
     <t>ASML US</t>
@@ -196,34 +217,13 @@
     <t>半导体设备</t>
   </si>
   <si>
-    <t>PWR US</t>
-  </si>
-  <si>
-    <t>广达服务</t>
-  </si>
-  <si>
-    <t>工程与建筑</t>
-  </si>
-  <si>
-    <t>WDAY US</t>
-  </si>
-  <si>
-    <t>Workday</t>
-  </si>
-  <si>
-    <t>MCHP US</t>
-  </si>
-  <si>
-    <t>微芯科技</t>
-  </si>
-  <si>
-    <t>半导体</t>
-  </si>
-  <si>
-    <t>NXPI US</t>
-  </si>
-  <si>
-    <t>恩智浦</t>
+    <t>MELI US</t>
+  </si>
+  <si>
+    <t>美客多</t>
+  </si>
+  <si>
+    <t>互联网零售</t>
   </si>
 </sst>
 </file>
@@ -573,9 +573,6 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I21"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
-  <cols>
-    <col min="9" max="9" width="9.5" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A1" t="s">
@@ -620,10 +617,10 @@
         <v>12</v>
       </c>
       <c r="E2">
-        <v>0.8</v>
+        <v>0.81</v>
       </c>
       <c r="F2">
-        <v>0.7</v>
+        <v>0.71</v>
       </c>
       <c r="G2" t="s">
         <v>13</v>
@@ -632,7 +629,7 @@
         <v>1.01</v>
       </c>
       <c r="I2" s="1">
-        <v>0.16120000000000001</v>
+        <v>0.15540000000000001</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.15">
@@ -649,10 +646,10 @@
         <v>16</v>
       </c>
       <c r="E3">
-        <v>0.81</v>
+        <v>0.84</v>
       </c>
       <c r="F3">
-        <v>0.71</v>
+        <v>0.74</v>
       </c>
       <c r="G3" t="s">
         <v>13</v>
@@ -661,7 +658,7 @@
         <v>1.01</v>
       </c>
       <c r="I3" s="1">
-        <v>0.15970000000000001</v>
+        <v>0.20119999999999999</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.15">
@@ -678,10 +675,10 @@
         <v>19</v>
       </c>
       <c r="E4">
-        <v>0.84</v>
+        <v>0.83</v>
       </c>
       <c r="F4">
-        <v>0.74</v>
+        <v>0.73</v>
       </c>
       <c r="G4" t="s">
         <v>13</v>
@@ -690,7 +687,7 @@
         <v>1.01</v>
       </c>
       <c r="I4" s="1">
-        <v>0.14879999999999999</v>
+        <v>0.14929999999999999</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.15">
@@ -719,7 +716,7 @@
         <v>1.01</v>
       </c>
       <c r="I5" s="1">
-        <v>0.15429999999999999</v>
+        <v>0.15279999999999999</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.15">
@@ -748,7 +745,7 @@
         <v>1.01</v>
       </c>
       <c r="I6" s="1">
-        <v>0.122</v>
+        <v>0.13189999999999999</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.15">
@@ -765,10 +762,10 @@
         <v>28</v>
       </c>
       <c r="E7">
-        <v>0.79</v>
+        <v>0.85</v>
       </c>
       <c r="F7">
-        <v>0.69</v>
+        <v>0.75</v>
       </c>
       <c r="G7" t="s">
         <v>13</v>
@@ -777,7 +774,7 @@
         <v>1.01</v>
       </c>
       <c r="I7" s="1">
-        <v>0.1535</v>
+        <v>0.20280000000000001</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.15">
@@ -794,10 +791,10 @@
         <v>32</v>
       </c>
       <c r="E8">
-        <v>0.83</v>
+        <v>0.85</v>
       </c>
       <c r="F8">
-        <v>0.73</v>
+        <v>0.75</v>
       </c>
       <c r="G8" t="s">
         <v>13</v>
@@ -806,7 +803,7 @@
         <v>1.01</v>
       </c>
       <c r="I8" s="1">
-        <v>0.19489999999999999</v>
+        <v>0.19689999999999999</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.15">
@@ -823,10 +820,10 @@
         <v>35</v>
       </c>
       <c r="E9">
-        <v>0.83</v>
+        <v>0.84</v>
       </c>
       <c r="F9">
-        <v>0.73</v>
+        <v>0.74</v>
       </c>
       <c r="G9" t="s">
         <v>13</v>
@@ -835,7 +832,7 @@
         <v>1.01</v>
       </c>
       <c r="I9" s="1">
-        <v>0.19520000000000001</v>
+        <v>0.1903</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.15">
@@ -852,10 +849,10 @@
         <v>38</v>
       </c>
       <c r="E10">
-        <v>0.82</v>
+        <v>0.83</v>
       </c>
       <c r="F10">
-        <v>0.72</v>
+        <v>0.73</v>
       </c>
       <c r="G10" t="s">
         <v>13</v>
@@ -864,7 +861,7 @@
         <v>1.01</v>
       </c>
       <c r="I10" s="1">
-        <v>0.20749999999999999</v>
+        <v>0.20080000000000001</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.15">
@@ -893,7 +890,7 @@
         <v>1.01</v>
       </c>
       <c r="I11" s="1">
-        <v>0.14419999999999999</v>
+        <v>0.1361</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.15">
@@ -910,10 +907,10 @@
         <v>28</v>
       </c>
       <c r="E12">
-        <v>0.84</v>
+        <v>0.85</v>
       </c>
       <c r="F12">
-        <v>0.74</v>
+        <v>0.75</v>
       </c>
       <c r="G12" t="s">
         <v>13</v>
@@ -922,7 +919,7 @@
         <v>1.01</v>
       </c>
       <c r="I12" s="1">
-        <v>0.14410000000000001</v>
+        <v>0.1426</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.15">
@@ -939,10 +936,10 @@
         <v>46</v>
       </c>
       <c r="E13">
-        <v>0.79</v>
+        <v>0.84</v>
       </c>
       <c r="F13">
-        <v>0.69</v>
+        <v>0.74</v>
       </c>
       <c r="G13" t="s">
         <v>13</v>
@@ -951,7 +948,7 @@
         <v>1.01</v>
       </c>
       <c r="I13" s="1">
-        <v>0.14799999999999999</v>
+        <v>0.20039999999999999</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.15">
@@ -980,7 +977,7 @@
         <v>1.01</v>
       </c>
       <c r="I14" s="1">
-        <v>0.1249</v>
+        <v>0.1855</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.15">
@@ -997,10 +994,10 @@
         <v>38</v>
       </c>
       <c r="E15">
-        <v>0.83</v>
+        <v>0.84</v>
       </c>
       <c r="F15">
-        <v>0.73</v>
+        <v>0.74</v>
       </c>
       <c r="G15" t="s">
         <v>13</v>
@@ -1009,7 +1006,7 @@
         <v>1.01</v>
       </c>
       <c r="I15" s="1">
-        <v>0.20180000000000001</v>
+        <v>0.20039999999999999</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.15">
@@ -1038,7 +1035,7 @@
         <v>1.01</v>
       </c>
       <c r="I16" s="1">
-        <v>0.12130000000000001</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.15">
@@ -1052,7 +1049,7 @@
         <v>56</v>
       </c>
       <c r="D17" t="s">
-        <v>57</v>
+        <v>22</v>
       </c>
       <c r="E17">
         <v>0.84</v>
@@ -1067,7 +1064,7 @@
         <v>1.01</v>
       </c>
       <c r="I17" s="1">
-        <v>0.13919999999999999</v>
+        <v>0.1429</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.15">
@@ -1075,19 +1072,19 @@
         <v>29</v>
       </c>
       <c r="B18" t="s">
+        <v>57</v>
+      </c>
+      <c r="C18" t="s">
         <v>58</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
         <v>59</v>
       </c>
-      <c r="D18" t="s">
-        <v>60</v>
-      </c>
       <c r="E18">
-        <v>0.85</v>
+        <v>0.82</v>
       </c>
       <c r="F18">
-        <v>0.75</v>
+        <v>0.72</v>
       </c>
       <c r="G18" t="s">
         <v>13</v>
@@ -1096,7 +1093,7 @@
         <v>1.01</v>
       </c>
       <c r="I18" s="1">
-        <v>0.13880000000000001</v>
+        <v>0.18840000000000001</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.15">
@@ -1104,19 +1101,19 @@
         <v>29</v>
       </c>
       <c r="B19" t="s">
+        <v>60</v>
+      </c>
+      <c r="C19" t="s">
         <v>61</v>
-      </c>
-      <c r="C19" t="s">
-        <v>62</v>
       </c>
       <c r="D19" t="s">
         <v>28</v>
       </c>
       <c r="E19">
-        <v>0.81</v>
+        <v>0.82</v>
       </c>
       <c r="F19">
-        <v>0.71</v>
+        <v>0.72</v>
       </c>
       <c r="G19" t="s">
         <v>13</v>
@@ -1125,7 +1122,7 @@
         <v>1.01</v>
       </c>
       <c r="I19" s="1">
-        <v>0.14180000000000001</v>
+        <v>0.14630000000000001</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.15">
@@ -1133,13 +1130,13 @@
         <v>29</v>
       </c>
       <c r="B20" t="s">
+        <v>62</v>
+      </c>
+      <c r="C20" t="s">
         <v>63</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
         <v>64</v>
-      </c>
-      <c r="D20" t="s">
-        <v>65</v>
       </c>
       <c r="E20">
         <v>0.85</v>
@@ -1154,7 +1151,7 @@
         <v>1.01</v>
       </c>
       <c r="I20" s="1">
-        <v>0.21440000000000001</v>
+        <v>0.12429999999999999</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.15">
@@ -1162,19 +1159,19 @@
         <v>29</v>
       </c>
       <c r="B21" t="s">
+        <v>65</v>
+      </c>
+      <c r="C21" t="s">
         <v>66</v>
       </c>
-      <c r="C21" t="s">
+      <c r="D21" t="s">
         <v>67</v>
       </c>
-      <c r="D21" t="s">
-        <v>65</v>
-      </c>
       <c r="E21">
-        <v>0.83</v>
+        <v>0.85</v>
       </c>
       <c r="F21">
-        <v>0.73</v>
+        <v>0.75</v>
       </c>
       <c r="G21" t="s">
         <v>13</v>
@@ -1183,7 +1180,7 @@
         <v>1.01</v>
       </c>
       <c r="I21" s="1">
-        <v>0.14899999999999999</v>
+        <v>0.1239</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
W43 2026 weekly update
- 本周标的+票息, 名称/行业自动中文, 热度榜5只IV<30替换(WBD/CVX/V/MA/1288→RCL/CoreWeave/安进/微软/礼来), 重生成 watchlist.json(58只)
- 财经日历刷新至W43(回顾ASML/台积电强劲·大行分化; 预告大型科技财报超级周TSLA/MSFT/谷歌/亚马逊·FOMC10/28)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/低波精选组.xlsx
+++ b/低波精选组.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Y:\GopherHK\Fixed Income\结构化产品\HTML 生成\FCN_Watchlist_交接\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29877FFB-46A7-4FE9-AE4B-FC95954F0F04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF0E6506-4AC3-4440-AACC-1E0044C225F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="69">
   <si>
     <t>区域</t>
   </si>
@@ -52,6 +52,18 @@
     <t>港股</t>
   </si>
   <si>
+    <t>1093 HK</t>
+  </si>
+  <si>
+    <t>石药集团</t>
+  </si>
+  <si>
+    <t>制药</t>
+  </si>
+  <si>
+    <t>欧式敲入</t>
+  </si>
+  <si>
     <t>2359 HK</t>
   </si>
   <si>
@@ -61,18 +73,6 @@
     <t>诊断与研究</t>
   </si>
   <si>
-    <t>欧式敲入</t>
-  </si>
-  <si>
-    <t>2269 HK</t>
-  </si>
-  <si>
-    <t>药明生物</t>
-  </si>
-  <si>
-    <t>生物科技</t>
-  </si>
-  <si>
     <t>2382 HK</t>
   </si>
   <si>
@@ -100,16 +100,76 @@
     <t>电商/云</t>
   </si>
   <si>
-    <t>20 HK</t>
-  </si>
-  <si>
-    <t>商汤-W</t>
+    <t>1810 HK</t>
+  </si>
+  <si>
+    <t>小米集团</t>
+  </si>
+  <si>
+    <t>AI/IoT</t>
+  </si>
+  <si>
+    <t>美股</t>
+  </si>
+  <si>
+    <t>PLTR US</t>
+  </si>
+  <si>
+    <t>帕兰提尔</t>
+  </si>
+  <si>
+    <t>AI软件</t>
+  </si>
+  <si>
+    <t>CRM US</t>
+  </si>
+  <si>
+    <t>赛富时</t>
   </si>
   <si>
     <t>应用软件</t>
   </si>
   <si>
-    <t>美股</t>
+    <t>ANET US</t>
+  </si>
+  <si>
+    <t>阿里斯塔</t>
+  </si>
+  <si>
+    <t>AI网络</t>
+  </si>
+  <si>
+    <t>META US</t>
+  </si>
+  <si>
+    <t>Meta平台</t>
+  </si>
+  <si>
+    <t>广告/AI</t>
+  </si>
+  <si>
+    <t>VLO US</t>
+  </si>
+  <si>
+    <t>瓦莱罗能源</t>
+  </si>
+  <si>
+    <t>油气炼化与销售</t>
+  </si>
+  <si>
+    <t>NOW US</t>
+  </si>
+  <si>
+    <t>ServiceNow</t>
+  </si>
+  <si>
+    <t>NEM US</t>
+  </si>
+  <si>
+    <t>纽曼矿业</t>
+  </si>
+  <si>
+    <t>黄金</t>
   </si>
   <si>
     <t>AMD US</t>
@@ -121,22 +181,25 @@
     <t>AI芯片</t>
   </si>
   <si>
-    <t>ANET US</t>
-  </si>
-  <si>
-    <t>阿里斯塔</t>
-  </si>
-  <si>
-    <t>AI网络</t>
-  </si>
-  <si>
-    <t>PLTR US</t>
-  </si>
-  <si>
-    <t>帕兰提尔</t>
-  </si>
-  <si>
-    <t>AI软件</t>
+    <t>DASH US</t>
+  </si>
+  <si>
+    <t>DoorDash</t>
+  </si>
+  <si>
+    <t>互联网零售</t>
+  </si>
+  <si>
+    <t>WDAY US</t>
+  </si>
+  <si>
+    <t>Workday</t>
+  </si>
+  <si>
+    <t>SPOT US</t>
+  </si>
+  <si>
+    <t>声田</t>
   </si>
   <si>
     <t>APH US</t>
@@ -148,66 +211,6 @@
     <t>电子元件</t>
   </si>
   <si>
-    <t>CRM US</t>
-  </si>
-  <si>
-    <t>赛富时</t>
-  </si>
-  <si>
-    <t>NU US</t>
-  </si>
-  <si>
-    <t>Nu控股</t>
-  </si>
-  <si>
-    <t>区域性银行</t>
-  </si>
-  <si>
-    <t>VLO US</t>
-  </si>
-  <si>
-    <t>瓦莱罗能源</t>
-  </si>
-  <si>
-    <t>油气炼化与销售</t>
-  </si>
-  <si>
-    <t>NOW US</t>
-  </si>
-  <si>
-    <t>ServiceNow</t>
-  </si>
-  <si>
-    <t>NEM US</t>
-  </si>
-  <si>
-    <t>纽曼矿业</t>
-  </si>
-  <si>
-    <t>黄金</t>
-  </si>
-  <si>
-    <t>SPOT US</t>
-  </si>
-  <si>
-    <t>声田</t>
-  </si>
-  <si>
-    <t>AMAT US</t>
-  </si>
-  <si>
-    <t>应用材料</t>
-  </si>
-  <si>
-    <t>半导体设备与材料</t>
-  </si>
-  <si>
-    <t>WDAY US</t>
-  </si>
-  <si>
-    <t>Workday</t>
-  </si>
-  <si>
     <t>ASML US</t>
   </si>
   <si>
@@ -217,13 +220,13 @@
     <t>半导体设备</t>
   </si>
   <si>
-    <t>MELI US</t>
-  </si>
-  <si>
-    <t>美客多</t>
-  </si>
-  <si>
-    <t>互联网零售</t>
+    <t>VST US</t>
+  </si>
+  <si>
+    <t>Vistra Energy</t>
+  </si>
+  <si>
+    <t>独立电力生产商</t>
   </si>
 </sst>
 </file>
@@ -617,10 +620,10 @@
         <v>12</v>
       </c>
       <c r="E2">
-        <v>0.81</v>
+        <v>0.83</v>
       </c>
       <c r="F2">
-        <v>0.71</v>
+        <v>0.73</v>
       </c>
       <c r="G2" t="s">
         <v>13</v>
@@ -629,7 +632,7 @@
         <v>1.01</v>
       </c>
       <c r="I2" s="1">
-        <v>0.15540000000000001</v>
+        <v>0.1628</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.15">
@@ -646,10 +649,10 @@
         <v>16</v>
       </c>
       <c r="E3">
-        <v>0.84</v>
+        <v>0.8</v>
       </c>
       <c r="F3">
-        <v>0.74</v>
+        <v>0.7</v>
       </c>
       <c r="G3" t="s">
         <v>13</v>
@@ -658,7 +661,7 @@
         <v>1.01</v>
       </c>
       <c r="I3" s="1">
-        <v>0.20119999999999999</v>
+        <v>0.17100000000000001</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.15">
@@ -704,10 +707,10 @@
         <v>22</v>
       </c>
       <c r="E5">
-        <v>0.82</v>
+        <v>0.81</v>
       </c>
       <c r="F5">
-        <v>0.72</v>
+        <v>0.71</v>
       </c>
       <c r="G5" t="s">
         <v>13</v>
@@ -716,7 +719,7 @@
         <v>1.01</v>
       </c>
       <c r="I5" s="1">
-        <v>0.15279999999999999</v>
+        <v>0.15609999999999999</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.15">
@@ -745,7 +748,7 @@
         <v>1.01</v>
       </c>
       <c r="I6" s="1">
-        <v>0.13189999999999999</v>
+        <v>0.1426</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.15">
@@ -762,10 +765,10 @@
         <v>28</v>
       </c>
       <c r="E7">
-        <v>0.85</v>
+        <v>0.84</v>
       </c>
       <c r="F7">
-        <v>0.75</v>
+        <v>0.74</v>
       </c>
       <c r="G7" t="s">
         <v>13</v>
@@ -774,7 +777,7 @@
         <v>1.01</v>
       </c>
       <c r="I7" s="1">
-        <v>0.20280000000000001</v>
+        <v>0.16020000000000001</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.15">
@@ -791,10 +794,10 @@
         <v>32</v>
       </c>
       <c r="E8">
-        <v>0.85</v>
+        <v>0.82</v>
       </c>
       <c r="F8">
-        <v>0.75</v>
+        <v>0.72</v>
       </c>
       <c r="G8" t="s">
         <v>13</v>
@@ -803,7 +806,7 @@
         <v>1.01</v>
       </c>
       <c r="I8" s="1">
-        <v>0.19689999999999999</v>
+        <v>0.2127</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.15">
@@ -832,7 +835,7 @@
         <v>1.01</v>
       </c>
       <c r="I9" s="1">
-        <v>0.1903</v>
+        <v>0.1416</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.15">
@@ -849,10 +852,10 @@
         <v>38</v>
       </c>
       <c r="E10">
-        <v>0.83</v>
+        <v>0.84</v>
       </c>
       <c r="F10">
-        <v>0.73</v>
+        <v>0.74</v>
       </c>
       <c r="G10" t="s">
         <v>13</v>
@@ -861,7 +864,7 @@
         <v>1.01</v>
       </c>
       <c r="I10" s="1">
-        <v>0.20080000000000001</v>
+        <v>0.19309999999999999</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.15">
@@ -878,10 +881,10 @@
         <v>41</v>
       </c>
       <c r="E11">
-        <v>0.84</v>
+        <v>0.85</v>
       </c>
       <c r="F11">
-        <v>0.74</v>
+        <v>0.75</v>
       </c>
       <c r="G11" t="s">
         <v>13</v>
@@ -890,7 +893,7 @@
         <v>1.01</v>
       </c>
       <c r="I11" s="1">
-        <v>0.1361</v>
+        <v>0.123</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.15">
@@ -904,13 +907,13 @@
         <v>43</v>
       </c>
       <c r="D12" t="s">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="E12">
-        <v>0.85</v>
+        <v>0.84</v>
       </c>
       <c r="F12">
-        <v>0.75</v>
+        <v>0.74</v>
       </c>
       <c r="G12" t="s">
         <v>13</v>
@@ -919,7 +922,7 @@
         <v>1.01</v>
       </c>
       <c r="I12" s="1">
-        <v>0.1426</v>
+        <v>0.18479999999999999</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.15">
@@ -927,19 +930,19 @@
         <v>29</v>
       </c>
       <c r="B13" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D13" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="E13">
-        <v>0.84</v>
+        <v>0.83</v>
       </c>
       <c r="F13">
-        <v>0.74</v>
+        <v>0.73</v>
       </c>
       <c r="G13" t="s">
         <v>13</v>
@@ -948,7 +951,7 @@
         <v>1.01</v>
       </c>
       <c r="I13" s="1">
-        <v>0.20039999999999999</v>
+        <v>0.2024</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.15">
@@ -977,7 +980,7 @@
         <v>1.01</v>
       </c>
       <c r="I14" s="1">
-        <v>0.1855</v>
+        <v>0.1087</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.15">
@@ -991,7 +994,7 @@
         <v>51</v>
       </c>
       <c r="D15" t="s">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="E15">
         <v>0.84</v>
@@ -1006,7 +1009,7 @@
         <v>1.01</v>
       </c>
       <c r="I15" s="1">
-        <v>0.20039999999999999</v>
+        <v>0.20130000000000001</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.15">
@@ -1014,13 +1017,13 @@
         <v>29</v>
       </c>
       <c r="B16" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C16" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D16" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E16">
         <v>0.85</v>
@@ -1035,7 +1038,7 @@
         <v>1.01</v>
       </c>
       <c r="I16" s="1">
-        <v>0.11</v>
+        <v>0.21279999999999999</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.15">
@@ -1043,19 +1046,19 @@
         <v>29</v>
       </c>
       <c r="B17" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C17" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D17" t="s">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="E17">
-        <v>0.84</v>
+        <v>0.83</v>
       </c>
       <c r="F17">
-        <v>0.74</v>
+        <v>0.73</v>
       </c>
       <c r="G17" t="s">
         <v>13</v>
@@ -1064,7 +1067,7 @@
         <v>1.01</v>
       </c>
       <c r="I17" s="1">
-        <v>0.1429</v>
+        <v>0.14530000000000001</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.15">
@@ -1072,19 +1075,19 @@
         <v>29</v>
       </c>
       <c r="B18" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C18" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D18" t="s">
-        <v>59</v>
+        <v>22</v>
       </c>
       <c r="E18">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="F18">
-        <v>0.72</v>
+        <v>0.75</v>
       </c>
       <c r="G18" t="s">
         <v>13</v>
@@ -1093,7 +1096,7 @@
         <v>1.01</v>
       </c>
       <c r="I18" s="1">
-        <v>0.18840000000000001</v>
+        <v>0.14460000000000001</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.15">
@@ -1107,13 +1110,13 @@
         <v>61</v>
       </c>
       <c r="D19" t="s">
-        <v>28</v>
+        <v>62</v>
       </c>
       <c r="E19">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="F19">
-        <v>0.72</v>
+        <v>0.75</v>
       </c>
       <c r="G19" t="s">
         <v>13</v>
@@ -1122,7 +1125,7 @@
         <v>1.01</v>
       </c>
       <c r="I19" s="1">
-        <v>0.14630000000000001</v>
+        <v>0.14030000000000001</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.15">
@@ -1130,13 +1133,13 @@
         <v>29</v>
       </c>
       <c r="B20" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C20" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D20" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E20">
         <v>0.85</v>
@@ -1151,7 +1154,7 @@
         <v>1.01</v>
       </c>
       <c r="I20" s="1">
-        <v>0.12429999999999999</v>
+        <v>0.1114</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.15">
@@ -1159,19 +1162,19 @@
         <v>29</v>
       </c>
       <c r="B21" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C21" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D21" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E21">
-        <v>0.85</v>
+        <v>0.81</v>
       </c>
       <c r="F21">
-        <v>0.75</v>
+        <v>0.71</v>
       </c>
       <c r="G21" t="s">
         <v>13</v>
@@ -1180,7 +1183,7 @@
         <v>1.01</v>
       </c>
       <c r="I21" s="1">
-        <v>0.1239</v>
+        <v>0.13600000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
W44 2026: watchlist.json + 三榜单Excel(上个commit漏提)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/低波精选组.xlsx
+++ b/低波精选组.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Y:\GopherHK\Fixed Income\结构化产品\HTML 生成\FCN_Watchlist_交接\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF0E6506-4AC3-4440-AACC-1E0044C225F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B30040B2-2EF5-48CD-9F40-A326C99C29B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="67">
   <si>
     <t>区域</t>
   </si>
@@ -91,6 +91,15 @@
     <t>互联网内容与信息</t>
   </si>
   <si>
+    <t>1810 HK</t>
+  </si>
+  <si>
+    <t>小米集团</t>
+  </si>
+  <si>
+    <t>AI/IoT</t>
+  </si>
+  <si>
     <t>9988 HK</t>
   </si>
   <si>
@@ -100,34 +109,88 @@
     <t>电商/云</t>
   </si>
   <si>
-    <t>1810 HK</t>
-  </si>
-  <si>
-    <t>小米集团</t>
-  </si>
-  <si>
-    <t>AI/IoT</t>
-  </si>
-  <si>
     <t>美股</t>
   </si>
   <si>
-    <t>PLTR US</t>
-  </si>
-  <si>
-    <t>帕兰提尔</t>
+    <t>CRM US</t>
+  </si>
+  <si>
+    <t>赛富时</t>
+  </si>
+  <si>
+    <t>应用软件</t>
+  </si>
+  <si>
+    <t>VLO US</t>
+  </si>
+  <si>
+    <t>瓦莱罗能源</t>
+  </si>
+  <si>
+    <t>油气炼化与销售</t>
+  </si>
+  <si>
+    <t>NOW US</t>
+  </si>
+  <si>
+    <t>ServiceNow</t>
   </si>
   <si>
     <t>AI软件</t>
   </si>
   <si>
-    <t>CRM US</t>
-  </si>
-  <si>
-    <t>赛富时</t>
-  </si>
-  <si>
-    <t>应用软件</t>
+    <t>AMD US</t>
+  </si>
+  <si>
+    <t>超微半导体</t>
+  </si>
+  <si>
+    <t>AI芯片</t>
+  </si>
+  <si>
+    <t>WDAY US</t>
+  </si>
+  <si>
+    <t>Workday</t>
+  </si>
+  <si>
+    <t>ADI US</t>
+  </si>
+  <si>
+    <t>亚德诺</t>
+  </si>
+  <si>
+    <t>半导体</t>
+  </si>
+  <si>
+    <t>SPOT US</t>
+  </si>
+  <si>
+    <t>声田</t>
+  </si>
+  <si>
+    <t>NU US</t>
+  </si>
+  <si>
+    <t>Nu控股</t>
+  </si>
+  <si>
+    <t>区域性银行</t>
+  </si>
+  <si>
+    <t>APH US</t>
+  </si>
+  <si>
+    <t>安费诺</t>
+  </si>
+  <si>
+    <t>电子元件</t>
+  </si>
+  <si>
+    <t>TXN US</t>
+  </si>
+  <si>
+    <t>德州仪器</t>
   </si>
   <si>
     <t>ANET US</t>
@@ -139,85 +202,16 @@
     <t>AI网络</t>
   </si>
   <si>
-    <t>META US</t>
-  </si>
-  <si>
-    <t>Meta平台</t>
-  </si>
-  <si>
-    <t>广告/AI</t>
-  </si>
-  <si>
-    <t>VLO US</t>
-  </si>
-  <si>
-    <t>瓦莱罗能源</t>
-  </si>
-  <si>
-    <t>油气炼化与销售</t>
-  </si>
-  <si>
-    <t>NOW US</t>
-  </si>
-  <si>
-    <t>ServiceNow</t>
-  </si>
-  <si>
-    <t>NEM US</t>
-  </si>
-  <si>
-    <t>纽曼矿业</t>
-  </si>
-  <si>
-    <t>黄金</t>
-  </si>
-  <si>
-    <t>AMD US</t>
-  </si>
-  <si>
-    <t>超微半导体</t>
-  </si>
-  <si>
-    <t>AI芯片</t>
-  </si>
-  <si>
-    <t>DASH US</t>
-  </si>
-  <si>
-    <t>DoorDash</t>
-  </si>
-  <si>
-    <t>互联网零售</t>
-  </si>
-  <si>
-    <t>WDAY US</t>
-  </si>
-  <si>
-    <t>Workday</t>
-  </si>
-  <si>
-    <t>SPOT US</t>
-  </si>
-  <si>
-    <t>声田</t>
-  </si>
-  <si>
-    <t>APH US</t>
-  </si>
-  <si>
-    <t>安费诺</t>
-  </si>
-  <si>
-    <t>电子元件</t>
-  </si>
-  <si>
-    <t>ASML US</t>
-  </si>
-  <si>
-    <t>阿斯麦</t>
-  </si>
-  <si>
-    <t>半导体设备</t>
+    <t>NXPI US</t>
+  </si>
+  <si>
+    <t>恩智浦</t>
+  </si>
+  <si>
+    <t>INTU US</t>
+  </si>
+  <si>
+    <t>财捷</t>
   </si>
   <si>
     <t>VST US</t>
@@ -620,10 +614,10 @@
         <v>12</v>
       </c>
       <c r="E2">
-        <v>0.83</v>
+        <v>0.82</v>
       </c>
       <c r="F2">
-        <v>0.73</v>
+        <v>0.72</v>
       </c>
       <c r="G2" t="s">
         <v>13</v>
@@ -632,7 +626,7 @@
         <v>1.01</v>
       </c>
       <c r="I2" s="1">
-        <v>0.1628</v>
+        <v>0.16120000000000001</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.15">
@@ -649,10 +643,10 @@
         <v>16</v>
       </c>
       <c r="E3">
-        <v>0.8</v>
+        <v>0.79</v>
       </c>
       <c r="F3">
-        <v>0.7</v>
+        <v>0.69</v>
       </c>
       <c r="G3" t="s">
         <v>13</v>
@@ -661,7 +655,7 @@
         <v>1.01</v>
       </c>
       <c r="I3" s="1">
-        <v>0.17100000000000001</v>
+        <v>0.17343</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.15">
@@ -690,7 +684,7 @@
         <v>1.01</v>
       </c>
       <c r="I4" s="1">
-        <v>0.14929999999999999</v>
+        <v>0.15240000000000001</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.15">
@@ -707,10 +701,10 @@
         <v>22</v>
       </c>
       <c r="E5">
-        <v>0.81</v>
+        <v>0.8</v>
       </c>
       <c r="F5">
-        <v>0.71</v>
+        <v>0.7</v>
       </c>
       <c r="G5" t="s">
         <v>13</v>
@@ -719,7 +713,7 @@
         <v>1.01</v>
       </c>
       <c r="I5" s="1">
-        <v>0.15609999999999999</v>
+        <v>0.15629999999999999</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.15">
@@ -736,10 +730,10 @@
         <v>25</v>
       </c>
       <c r="E6">
-        <v>0.85</v>
+        <v>0.84</v>
       </c>
       <c r="F6">
-        <v>0.75</v>
+        <v>0.74</v>
       </c>
       <c r="G6" t="s">
         <v>13</v>
@@ -748,7 +742,7 @@
         <v>1.01</v>
       </c>
       <c r="I6" s="1">
-        <v>0.1426</v>
+        <v>0.16309999999999999</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.15">
@@ -765,10 +759,10 @@
         <v>28</v>
       </c>
       <c r="E7">
-        <v>0.84</v>
+        <v>0.85</v>
       </c>
       <c r="F7">
-        <v>0.74</v>
+        <v>0.75</v>
       </c>
       <c r="G7" t="s">
         <v>13</v>
@@ -777,7 +771,7 @@
         <v>1.01</v>
       </c>
       <c r="I7" s="1">
-        <v>0.16020000000000001</v>
+        <v>0.15010000000000001</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.15">
@@ -794,10 +788,10 @@
         <v>32</v>
       </c>
       <c r="E8">
-        <v>0.82</v>
+        <v>0.83</v>
       </c>
       <c r="F8">
-        <v>0.72</v>
+        <v>0.73</v>
       </c>
       <c r="G8" t="s">
         <v>13</v>
@@ -806,7 +800,7 @@
         <v>1.01</v>
       </c>
       <c r="I8" s="1">
-        <v>0.2127</v>
+        <v>0.14630000000000001</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.15">
@@ -835,7 +829,7 @@
         <v>1.01</v>
       </c>
       <c r="I9" s="1">
-        <v>0.1416</v>
+        <v>0.1966</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.15">
@@ -852,10 +846,10 @@
         <v>38</v>
       </c>
       <c r="E10">
-        <v>0.84</v>
+        <v>0.82</v>
       </c>
       <c r="F10">
-        <v>0.74</v>
+        <v>0.72</v>
       </c>
       <c r="G10" t="s">
         <v>13</v>
@@ -864,7 +858,7 @@
         <v>1.01</v>
       </c>
       <c r="I10" s="1">
-        <v>0.19309999999999999</v>
+        <v>0.2009</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.15">
@@ -881,10 +875,10 @@
         <v>41</v>
       </c>
       <c r="E11">
-        <v>0.85</v>
+        <v>0.81</v>
       </c>
       <c r="F11">
-        <v>0.75</v>
+        <v>0.71</v>
       </c>
       <c r="G11" t="s">
         <v>13</v>
@@ -893,7 +887,7 @@
         <v>1.01</v>
       </c>
       <c r="I11" s="1">
-        <v>0.123</v>
+        <v>0.1981</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.15">
@@ -907,7 +901,7 @@
         <v>43</v>
       </c>
       <c r="D12" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="E12">
         <v>0.84</v>
@@ -922,7 +916,7 @@
         <v>1.01</v>
       </c>
       <c r="I12" s="1">
-        <v>0.18479999999999999</v>
+        <v>0.1358</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.15">
@@ -930,19 +924,19 @@
         <v>29</v>
       </c>
       <c r="B13" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13" t="s">
         <v>45</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>46</v>
       </c>
-      <c r="D13" t="s">
-        <v>32</v>
-      </c>
       <c r="E13">
-        <v>0.83</v>
+        <v>0.85</v>
       </c>
       <c r="F13">
-        <v>0.73</v>
+        <v>0.75</v>
       </c>
       <c r="G13" t="s">
         <v>13</v>
@@ -951,7 +945,7 @@
         <v>1.01</v>
       </c>
       <c r="I13" s="1">
-        <v>0.2024</v>
+        <v>0.14530000000000001</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.15">
@@ -965,7 +959,7 @@
         <v>48</v>
       </c>
       <c r="D14" t="s">
-        <v>49</v>
+        <v>22</v>
       </c>
       <c r="E14">
         <v>0.85</v>
@@ -980,7 +974,7 @@
         <v>1.01</v>
       </c>
       <c r="I14" s="1">
-        <v>0.1087</v>
+        <v>0.12759999999999999</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.15">
@@ -988,19 +982,19 @@
         <v>29</v>
       </c>
       <c r="B15" t="s">
+        <v>49</v>
+      </c>
+      <c r="C15" t="s">
         <v>50</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
         <v>51</v>
       </c>
-      <c r="D15" t="s">
-        <v>52</v>
-      </c>
       <c r="E15">
-        <v>0.84</v>
+        <v>0.79</v>
       </c>
       <c r="F15">
-        <v>0.74</v>
+        <v>0.69</v>
       </c>
       <c r="G15" t="s">
         <v>13</v>
@@ -1009,7 +1003,7 @@
         <v>1.01</v>
       </c>
       <c r="I15" s="1">
-        <v>0.20130000000000001</v>
+        <v>0.1293</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.15">
@@ -1017,19 +1011,19 @@
         <v>29</v>
       </c>
       <c r="B16" t="s">
+        <v>52</v>
+      </c>
+      <c r="C16" t="s">
         <v>53</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
         <v>54</v>
       </c>
-      <c r="D16" t="s">
-        <v>55</v>
-      </c>
       <c r="E16">
-        <v>0.85</v>
+        <v>0.82</v>
       </c>
       <c r="F16">
-        <v>0.75</v>
+        <v>0.72</v>
       </c>
       <c r="G16" t="s">
         <v>13</v>
@@ -1038,7 +1032,7 @@
         <v>1.01</v>
       </c>
       <c r="I16" s="1">
-        <v>0.21279999999999999</v>
+        <v>0.14169999999999999</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.15">
@@ -1046,19 +1040,19 @@
         <v>29</v>
       </c>
       <c r="B17" t="s">
+        <v>55</v>
+      </c>
+      <c r="C17" t="s">
         <v>56</v>
       </c>
-      <c r="C17" t="s">
-        <v>57</v>
-      </c>
       <c r="D17" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="E17">
-        <v>0.83</v>
+        <v>0.85</v>
       </c>
       <c r="F17">
-        <v>0.73</v>
+        <v>0.75</v>
       </c>
       <c r="G17" t="s">
         <v>13</v>
@@ -1067,7 +1061,7 @@
         <v>1.01</v>
       </c>
       <c r="I17" s="1">
-        <v>0.14530000000000001</v>
+        <v>0.13819999999999999</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.15">
@@ -1075,19 +1069,19 @@
         <v>29</v>
       </c>
       <c r="B18" t="s">
+        <v>57</v>
+      </c>
+      <c r="C18" t="s">
         <v>58</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
         <v>59</v>
       </c>
-      <c r="D18" t="s">
-        <v>22</v>
-      </c>
       <c r="E18">
-        <v>0.85</v>
+        <v>0.82</v>
       </c>
       <c r="F18">
-        <v>0.75</v>
+        <v>0.72</v>
       </c>
       <c r="G18" t="s">
         <v>13</v>
@@ -1096,7 +1090,7 @@
         <v>1.01</v>
       </c>
       <c r="I18" s="1">
-        <v>0.14460000000000001</v>
+        <v>0.2016</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.15">
@@ -1110,13 +1104,13 @@
         <v>61</v>
       </c>
       <c r="D19" t="s">
-        <v>62</v>
+        <v>46</v>
       </c>
       <c r="E19">
-        <v>0.85</v>
+        <v>0.81</v>
       </c>
       <c r="F19">
-        <v>0.75</v>
+        <v>0.71</v>
       </c>
       <c r="G19" t="s">
         <v>13</v>
@@ -1125,7 +1119,7 @@
         <v>1.01</v>
       </c>
       <c r="I19" s="1">
-        <v>0.14030000000000001</v>
+        <v>0.1472</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.15">
@@ -1133,19 +1127,19 @@
         <v>29</v>
       </c>
       <c r="B20" t="s">
+        <v>62</v>
+      </c>
+      <c r="C20" t="s">
         <v>63</v>
       </c>
-      <c r="C20" t="s">
-        <v>64</v>
-      </c>
       <c r="D20" t="s">
-        <v>65</v>
+        <v>32</v>
       </c>
       <c r="E20">
-        <v>0.85</v>
+        <v>0.84</v>
       </c>
       <c r="F20">
-        <v>0.75</v>
+        <v>0.74</v>
       </c>
       <c r="G20" t="s">
         <v>13</v>
@@ -1154,7 +1148,7 @@
         <v>1.01</v>
       </c>
       <c r="I20" s="1">
-        <v>0.1114</v>
+        <v>0.19769999999999999</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.15">
@@ -1162,19 +1156,19 @@
         <v>29</v>
       </c>
       <c r="B21" t="s">
+        <v>64</v>
+      </c>
+      <c r="C21" t="s">
+        <v>65</v>
+      </c>
+      <c r="D21" t="s">
         <v>66</v>
       </c>
-      <c r="C21" t="s">
-        <v>67</v>
-      </c>
-      <c r="D21" t="s">
-        <v>68</v>
-      </c>
       <c r="E21">
-        <v>0.81</v>
+        <v>0.8</v>
       </c>
       <c r="F21">
-        <v>0.71</v>
+        <v>0.7</v>
       </c>
       <c r="G21" t="s">
         <v>13</v>
@@ -1183,7 +1177,7 @@
         <v>1.01</v>
       </c>
       <c r="I21" s="1">
-        <v>0.13600000000000001</v>
+        <v>0.1525</v>
       </c>
     </row>
   </sheetData>

</xml_diff>